<commit_message>
update TC AML sàng lọc
</commit_message>
<xml_diff>
--- a/practices/testcases/msb-aml-tf/api/TC_AML_TRANSACTION_SCREENING_API 4.xlsx
+++ b/practices/testcases/msb-aml-tf/api/TC_AML_TRANSACTION_SCREENING_API 4.xlsx
@@ -545,6 +545,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:S387"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -686,7 +689,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
+    <row r="3" xml:space="preserve" outlineLevel="1">
       <c r="A3" s="5" t="str">
         <v>AML_API_EP_01</v>
       </c>
@@ -774,7 +777,7 @@
         <v>TD: TD_P1_001 | [GIU NGUYEN] ID goc: AML_API_EP_01</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
+    <row r="4" xml:space="preserve" outlineLevel="1">
       <c r="A4" s="5" t="str">
         <v>AML_API_HDR_01</v>
       </c>
@@ -862,7 +865,7 @@
         <v>TD: TD_P1_002 | [GIU NGUYEN] ID goc: AML_API_HDR_01</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
+    <row r="5" xml:space="preserve" outlineLevel="1">
       <c r="A5" s="5" t="str">
         <v>AML_API_NF_08</v>
       </c>
@@ -939,7 +942,7 @@
         <v>TD: TD_P2_001 | [GIU NGUYEN] ID goc: AML_API_NF_08</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
+    <row r="6" xml:space="preserve" outlineLevel="1">
       <c r="A6" s="5" t="str">
         <v>AML_API_NF_01</v>
       </c>
@@ -1022,7 +1025,7 @@
         <v>TD: TD_P3_005 | [GIU NGUYEN] ID goc: AML_API_NF_01</v>
       </c>
     </row>
-    <row r="7" xml:space="preserve">
+    <row r="7" xml:space="preserve" outlineLevel="1">
       <c r="A7" s="5" t="str">
         <v/>
       </c>
@@ -1103,7 +1106,7 @@
         <v>TD: TD_P3_006 | [TC MOI THEM] [BVA+] | Ly do: TC goc chi co case bien tren hop le cho channel (AML_API_NF_01), chua co cho transactionId</v>
       </c>
     </row>
-    <row r="8" xml:space="preserve">
+    <row r="8" xml:space="preserve" outlineLevel="1">
       <c r="A8" s="5" t="str">
         <v/>
       </c>
@@ -1184,7 +1187,7 @@
         <v>TD: TD_P3_007 | [TC MOI THEM] [BVA+] | Ly do: TC goc chi co case bien tren hop le cho channel, chua co cho requestId</v>
       </c>
     </row>
-    <row r="9" xml:space="preserve">
+    <row r="9" xml:space="preserve" outlineLevel="1">
       <c r="A9" s="5" t="str">
         <v/>
       </c>
@@ -1265,7 +1268,7 @@
         <v>TD: TD_P3_008 | [TC MOI THEM] [BVA+] | Ly do: TC goc chi co case bien tren hop le cho channel, chua co cho branchCd</v>
       </c>
     </row>
-    <row r="10" xml:space="preserve">
+    <row r="10" xml:space="preserve" outlineLevel="1">
       <c r="A10" s="5" t="str">
         <v>AML_API_NF_06</v>
       </c>
@@ -1410,7 +1413,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" xml:space="preserve">
+    <row r="12" xml:space="preserve" outlineLevel="1">
       <c r="A12" s="5" t="str">
         <v>AML_API_MT_01</v>
       </c>
@@ -1500,7 +1503,7 @@
         <v>TD: TD_P3_013 | [GIU NGUYEN] ID goc: AML_API_MT_01</v>
       </c>
     </row>
-    <row r="13" xml:space="preserve">
+    <row r="13" xml:space="preserve" outlineLevel="1">
       <c r="A13" s="5" t="str">
         <v>AML_API_MT_02</v>
       </c>
@@ -1590,7 +1593,7 @@
         <v>TD: TD_P3_014 | [GIU NGUYEN] ID goc: AML_API_MT_02</v>
       </c>
     </row>
-    <row r="14" xml:space="preserve">
+    <row r="14" xml:space="preserve" outlineLevel="1">
       <c r="A14" s="5" t="str">
         <v>AML_API_MT_03</v>
       </c>
@@ -1741,7 +1744,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" xml:space="preserve">
+    <row r="16" xml:space="preserve" outlineLevel="1">
       <c r="A16" s="5" t="str">
         <v>AML_API_MX_01</v>
       </c>
@@ -1854,7 +1857,7 @@
         <v>TD: TD_P3_018 | [GIU NGUYEN] ID goc: AML_API_MX_01</v>
       </c>
     </row>
-    <row r="17" xml:space="preserve">
+    <row r="17" xml:space="preserve" outlineLevel="1">
       <c r="A17" s="5" t="str">
         <v>AML_API_MX_02</v>
       </c>
@@ -1967,7 +1970,7 @@
         <v>TD: TD_P3_019 | [GIU NGUYEN] ID goc: AML_API_MX_02</v>
       </c>
     </row>
-    <row r="18" xml:space="preserve">
+    <row r="18" xml:space="preserve" outlineLevel="1">
       <c r="A18" s="5" t="str">
         <v>AML_API_MX_03</v>
       </c>
@@ -2080,7 +2083,7 @@
         <v>TD: TD_P3_020 | [GIU NGUYEN] ID goc: AML_API_MX_03</v>
       </c>
     </row>
-    <row r="19" xml:space="preserve">
+    <row r="19" xml:space="preserve" outlineLevel="1">
       <c r="A19" s="5" t="str">
         <v>AML_API_MX_04</v>
       </c>
@@ -2402,7 +2405,7 @@
         <v>TD: TD_P3_021 | [GIU NGUYEN] ID goc: AML_API_MX_04</v>
       </c>
     </row>
-    <row r="20" xml:space="preserve">
+    <row r="20" xml:space="preserve" outlineLevel="1">
       <c r="A20" s="5" t="str">
         <v>AML_API_MX_06</v>
       </c>
@@ -2548,7 +2551,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" xml:space="preserve">
+    <row r="22" xml:space="preserve" outlineLevel="1">
       <c r="A22" s="5" t="str">
         <v>AML_API_MSB001_01</v>
       </c>
@@ -2646,7 +2649,7 @@
         <v>TD: TD_P3_023 | [GIU NGUYEN] ID goc: AML_API_MSB001_01</v>
       </c>
     </row>
-    <row r="23" xml:space="preserve">
+    <row r="23" xml:space="preserve" outlineLevel="1">
       <c r="A23" s="5" t="str">
         <v>AML_API_MSB001_02</v>
       </c>
@@ -2737,7 +2740,7 @@
         <v>TD: TD_P3_024 | [GIU NGUYEN] ID goc: AML_API_MSB001_02</v>
       </c>
     </row>
-    <row r="24" xml:space="preserve">
+    <row r="24" xml:space="preserve" outlineLevel="1">
       <c r="A24" s="5" t="str">
         <v>AML_API_MSB001_03</v>
       </c>
@@ -2895,7 +2898,7 @@
         <v>TD: TD_P3_025 | [GIU NGUYEN] ID goc: AML_API_MSB001_03</v>
       </c>
     </row>
-    <row r="25" xml:space="preserve">
+    <row r="25" xml:space="preserve" outlineLevel="1">
       <c r="A25" s="5" t="str">
         <v>AML_API_MSB001_05</v>
       </c>
@@ -2970,7 +2973,7 @@
         <v>TD: TD_P3_026 | [GIU NGUYEN] ID goc: AML_API_MSB001_05</v>
       </c>
     </row>
-    <row r="26" xml:space="preserve">
+    <row r="26" xml:space="preserve" outlineLevel="1">
       <c r="A26" s="5" t="str">
         <v>AML_MSB001_MND_01</v>
       </c>
@@ -3096,7 +3099,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" xml:space="preserve">
+    <row r="28" xml:space="preserve" outlineLevel="1">
       <c r="A28" s="5" t="str">
         <v>AML_API_MSB002_01</v>
       </c>
@@ -3254,7 +3257,7 @@
         <v>TD: TD_P3_028 | [GIU NGUYEN] ID goc: AML_API_MSB002_01</v>
       </c>
     </row>
-    <row r="29" xml:space="preserve">
+    <row r="29" xml:space="preserve" outlineLevel="1">
       <c r="A29" s="5" t="str">
         <v>AML_API_MSB002_02</v>
       </c>
@@ -3345,7 +3348,7 @@
         <v>TD: TD_P3_029 | [GIU NGUYEN] ID goc: AML_API_MSB002_02</v>
       </c>
     </row>
-    <row r="30" xml:space="preserve">
+    <row r="30" xml:space="preserve" outlineLevel="1">
       <c r="A30" s="5" t="str">
         <v>AML_API_MSB002_03</v>
       </c>
@@ -3425,7 +3428,7 @@
         <v>TD: TD_P3_030 | [GIU NGUYEN] ID goc: AML_API_MSB002_03</v>
       </c>
     </row>
-    <row r="31" xml:space="preserve">
+    <row r="31" xml:space="preserve" outlineLevel="1">
       <c r="A31" s="5" t="str">
         <v>AML_API_NF_07</v>
       </c>
@@ -3512,7 +3515,7 @@
         <v>TD: TD_P3_031 | [GIU NGUYEN] ID goc: AML_API_NF_07</v>
       </c>
     </row>
-    <row r="32" xml:space="preserve">
+    <row r="32" xml:space="preserve" outlineLevel="1">
       <c r="A32" s="5" t="str">
         <v>AML_MSB002_MND_01</v>
       </c>
@@ -3638,7 +3641,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" xml:space="preserve">
+    <row r="34" xml:space="preserve" outlineLevel="1">
       <c r="A34" s="5" t="str">
         <v>AML_API_MSB003_01</v>
       </c>
@@ -3893,7 +3896,7 @@
         <v>TD: TD_P3_033 | [GIU NGUYEN] ID goc: AML_API_MSB003_01</v>
       </c>
     </row>
-    <row r="35" xml:space="preserve">
+    <row r="35" xml:space="preserve" outlineLevel="1">
       <c r="A35" s="5" t="str">
         <v>AML_API_MSB003_02</v>
       </c>
@@ -3982,7 +3985,7 @@
         <v>TD: TD_P3_034 | [GIU NGUYEN] ID goc: AML_API_MSB003_02</v>
       </c>
     </row>
-    <row r="36" xml:space="preserve">
+    <row r="36" xml:space="preserve" outlineLevel="1">
       <c r="A36" s="5" t="str">
         <v>AML_API_MSB003_03</v>
       </c>
@@ -4237,7 +4240,7 @@
         <v>TD: TD_P3_035 | [GIU NGUYEN] ID goc: AML_API_MSB003_03</v>
       </c>
     </row>
-    <row r="37" xml:space="preserve">
+    <row r="37" xml:space="preserve" outlineLevel="1">
       <c r="A37" s="5" t="str">
         <v>AML_MSB003_MND_01</v>
       </c>
@@ -4363,7 +4366,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" xml:space="preserve">
+    <row r="39" xml:space="preserve" outlineLevel="1">
       <c r="A39" s="5" t="str">
         <v>AML_API_EP_02</v>
       </c>
@@ -4431,7 +4434,7 @@
         <v>TD: TD_P1_003 | [GIU NGUYEN] ID goc: AML_API_EP_02</v>
       </c>
     </row>
-    <row r="40" xml:space="preserve">
+    <row r="40" xml:space="preserve" outlineLevel="1">
       <c r="A40" s="5" t="str">
         <v>AML_API_HTTP_04</v>
       </c>
@@ -4499,7 +4502,7 @@
         <v>TD: TD_P1_003 | [GIU NGUYEN] ID goc: AML_API_HTTP_04</v>
       </c>
     </row>
-    <row r="41" xml:space="preserve">
+    <row r="41" xml:space="preserve" outlineLevel="1">
       <c r="A41" s="5" t="str">
         <v>AML_API_EP_03</v>
       </c>
@@ -4567,7 +4570,7 @@
         <v>TD: TD_P1_004 | [GIU NGUYEN] ID goc: AML_API_EP_03</v>
       </c>
     </row>
-    <row r="42" xml:space="preserve">
+    <row r="42" xml:space="preserve" outlineLevel="1">
       <c r="A42" s="5" t="str">
         <v/>
       </c>
@@ -4643,7 +4646,7 @@
         <v>TD: TD_P1_005 | [TC MOI THEM] [Format] | Ly do: PTTK quy dinh Content-Type: application/json nhung TC goc chua co case sai Content-Type</v>
       </c>
     </row>
-    <row r="43" xml:space="preserve">
+    <row r="43" xml:space="preserve" outlineLevel="1">
       <c r="A43" s="5" t="str">
         <v/>
       </c>
@@ -4777,7 +4780,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" xml:space="preserve">
+    <row r="45" xml:space="preserve" outlineLevel="1">
       <c r="A45" s="5" t="str">
         <v>AML_API_HDR_02</v>
       </c>
@@ -4865,7 +4868,7 @@
         <v>TD: TD_P1_007 | [GIU NGUYEN] ID goc: AML_API_HDR_02</v>
       </c>
     </row>
-    <row r="46" xml:space="preserve">
+    <row r="46" xml:space="preserve" outlineLevel="1">
       <c r="A46" s="5" t="str">
         <v/>
       </c>
@@ -4950,7 +4953,7 @@
         <v>TD: TD_P1_016 | [TC MOI THEM] [Basic] | Ly do: TC goc chi co case THIEU HAN header (AML_API_HDR_02), chua tach case truyen gia tri rong</v>
       </c>
     </row>
-    <row r="47" xml:space="preserve">
+    <row r="47" xml:space="preserve" outlineLevel="1">
       <c r="A47" s="5" t="str">
         <v>AML_API_HDR_12</v>
       </c>
@@ -5031,7 +5034,7 @@
         <v>TD: TD_P2_002 | [GIU NGUYEN] ID goc: AML_API_HDR_12</v>
       </c>
     </row>
-    <row r="48" xml:space="preserve">
+    <row r="48" xml:space="preserve" outlineLevel="1">
       <c r="A48" s="5" t="str">
         <v>AML_API_NF_03</v>
       </c>
@@ -5168,7 +5171,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" xml:space="preserve">
+    <row r="50" xml:space="preserve" outlineLevel="1">
       <c r="A50" s="5" t="str">
         <v>AML_API_HDR_03</v>
       </c>
@@ -5256,7 +5259,7 @@
         <v>TD: TD_P1_008 | [GIU NGUYEN] ID goc: AML_API_HDR_03</v>
       </c>
     </row>
-    <row r="51" xml:space="preserve">
+    <row r="51" xml:space="preserve" outlineLevel="1">
       <c r="A51" s="5" t="str">
         <v/>
       </c>
@@ -5399,7 +5402,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" xml:space="preserve">
+    <row r="53" xml:space="preserve" outlineLevel="1">
       <c r="A53" s="5" t="str">
         <v>AML_API_HDR_04</v>
       </c>
@@ -5487,7 +5490,7 @@
         <v>TD: TD_P1_009 | [GIU NGUYEN] ID goc: AML_API_HDR_04</v>
       </c>
     </row>
-    <row r="54" xml:space="preserve">
+    <row r="54" xml:space="preserve" outlineLevel="1">
       <c r="A54" s="5" t="str">
         <v>AML_API_HDR_13</v>
       </c>
@@ -5575,7 +5578,7 @@
         <v>TD: TD_P1_015 | [GIU NGUYEN] ID goc: AML_API_HDR_13</v>
       </c>
     </row>
-    <row r="55" xml:space="preserve">
+    <row r="55" xml:space="preserve" outlineLevel="1">
       <c r="A55" s="5" t="str">
         <v/>
       </c>
@@ -5718,7 +5721,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" xml:space="preserve">
+    <row r="57" xml:space="preserve" outlineLevel="1">
       <c r="A57" s="5" t="str">
         <v>AML_API_HDR_05</v>
       </c>
@@ -5806,7 +5809,7 @@
         <v>TD: TD_P1_010 | [GIU NGUYEN] ID goc: AML_API_HDR_05</v>
       </c>
     </row>
-    <row r="58" xml:space="preserve">
+    <row r="58" xml:space="preserve" outlineLevel="1">
       <c r="A58" s="5" t="str">
         <v/>
       </c>
@@ -5949,7 +5952,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" xml:space="preserve">
+    <row r="60" xml:space="preserve" outlineLevel="1">
       <c r="A60" s="5" t="str">
         <v>AML_API_HDR_06</v>
       </c>
@@ -6037,7 +6040,7 @@
         <v>TD: TD_P1_011 | [GIU NGUYEN] ID goc: AML_API_HDR_06</v>
       </c>
     </row>
-    <row r="61" xml:space="preserve">
+    <row r="61" xml:space="preserve" outlineLevel="1">
       <c r="A61" s="5" t="str">
         <v>AML_API_NF_02</v>
       </c>
@@ -6124,7 +6127,7 @@
         <v>TD: TD_P2_003 | [GIU NGUYEN] ID goc: AML_API_NF_02</v>
       </c>
     </row>
-    <row r="62" xml:space="preserve">
+    <row r="62" xml:space="preserve" outlineLevel="1">
       <c r="A62" s="5" t="str">
         <v/>
       </c>
@@ -6202,7 +6205,7 @@
         <v>TD: TD_P3_010 | [TC MOI THEM] [EG] | Ly do: Error Guessing cho field Text tu do - TC goc chi kiem ky tu dac biet trong transactionId (AML_API_NF_03)</v>
       </c>
     </row>
-    <row r="63" xml:space="preserve">
+    <row r="63" xml:space="preserve" outlineLevel="1">
       <c r="A63" s="5" t="str">
         <v/>
       </c>
@@ -6338,7 +6341,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" xml:space="preserve">
+    <row r="65" xml:space="preserve" outlineLevel="1">
       <c r="A65" s="5" t="str">
         <v>AML_API_HDR_07</v>
       </c>
@@ -6420,7 +6423,7 @@
         <v>TD: TD_P1_012 | [GIU NGUYEN] ID goc: AML_API_HDR_07</v>
       </c>
     </row>
-    <row r="66" xml:space="preserve">
+    <row r="66" xml:space="preserve" outlineLevel="1">
       <c r="A66" s="5" t="str">
         <v>AML_API_HDR_11</v>
       </c>
@@ -6567,7 +6570,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" xml:space="preserve">
+    <row r="68" xml:space="preserve" outlineLevel="1">
       <c r="A68" s="5" t="str">
         <v>AML_API_HDR_08</v>
       </c>
@@ -6655,7 +6658,7 @@
         <v>TD: TD_P1_013 | [GIU NGUYEN] ID goc: AML_API_HDR_08</v>
       </c>
     </row>
-    <row r="69" xml:space="preserve">
+    <row r="69" xml:space="preserve" outlineLevel="1">
       <c r="A69" s="5" t="str">
         <v/>
       </c>
@@ -6798,7 +6801,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" xml:space="preserve">
+    <row r="71" xml:space="preserve" outlineLevel="1">
       <c r="A71" s="5" t="str">
         <v/>
       </c>
@@ -6940,7 +6943,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" xml:space="preserve">
+    <row r="73" xml:space="preserve" outlineLevel="1">
       <c r="A73" s="5" t="str">
         <v>AML_API_MT_04</v>
       </c>
@@ -7019,7 +7022,7 @@
         <v>TD: TD_P2_009 | [GIU NGUYEN] ID goc: AML_API_MT_04</v>
       </c>
     </row>
-    <row r="74" xml:space="preserve">
+    <row r="74" xml:space="preserve" outlineLevel="1">
       <c r="A74" s="5" t="str">
         <v>AML_API_MT_05</v>
       </c>
@@ -7150,7 +7153,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" xml:space="preserve">
+    <row r="76" xml:space="preserve" outlineLevel="1">
       <c r="A76" s="5" t="str">
         <v>AML_API_MX_05</v>
       </c>
@@ -7226,7 +7229,7 @@
         <v>TD: TD_P2_031 | [GIU NGUYEN] ID goc: AML_API_MX_05</v>
       </c>
     </row>
-    <row r="77" xml:space="preserve">
+    <row r="77" xml:space="preserve" outlineLevel="1">
       <c r="A77" s="5" t="str">
         <v>AML_API_MX_06</v>
       </c>
@@ -7357,7 +7360,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" xml:space="preserve">
+    <row r="79" xml:space="preserve" outlineLevel="1">
       <c r="A79" s="5" t="str">
         <v>AML_API_MSB001_04</v>
       </c>
@@ -7433,7 +7436,7 @@
         <v>TD: TD_P2_038 | [GIU NGUYEN] ID goc: AML_API_MSB001_04</v>
       </c>
     </row>
-    <row r="80" xml:space="preserve">
+    <row r="80" xml:space="preserve" outlineLevel="1">
       <c r="A80" s="5" t="str">
         <v/>
       </c>
@@ -7562,7 +7565,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" xml:space="preserve">
+    <row r="82" xml:space="preserve" outlineLevel="1">
       <c r="A82" s="5" t="str">
         <v>AML_API_MSB002_04</v>
       </c>
@@ -7637,7 +7640,7 @@
         <v>TD: TD_P2_041 | [GIU NGUYEN] ID goc: AML_API_MSB002_04</v>
       </c>
     </row>
-    <row r="83" xml:space="preserve">
+    <row r="83" xml:space="preserve" outlineLevel="1">
       <c r="A83" s="5" t="str">
         <v/>
       </c>
@@ -7766,7 +7769,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" xml:space="preserve">
+    <row r="85" xml:space="preserve" outlineLevel="1">
       <c r="A85" s="5" t="str">
         <v>AML_API_MSB003_04</v>
       </c>
@@ -8023,7 +8026,7 @@
         <v>TD: TD_P2_044 | [GIU NGUYEN] ID goc: AML_API_MSB003_04</v>
       </c>
     </row>
-    <row r="86" xml:space="preserve">
+    <row r="86" xml:space="preserve" outlineLevel="1">
       <c r="A86" s="5" t="str">
         <v/>
       </c>
@@ -8093,7 +8096,7 @@
         <v>TD: TD_P2_045 | [TC MOI THEM] [Malformed] | Ly do: TC goc co case JSON Object thay vi Array (AML_API_MSB003_04) nhung chua co case JSON sai cu phap</v>
       </c>
     </row>
-    <row r="87" xml:space="preserve">
+    <row r="87" xml:space="preserve" outlineLevel="1">
       <c r="A87" s="5" t="str">
         <v/>
       </c>
@@ -8222,7 +8225,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" xml:space="preserve">
+    <row r="89" xml:space="preserve" outlineLevel="1">
       <c r="A89" s="5" t="str">
         <v>AML_MT195_MND_01</v>
       </c>
@@ -8300,7 +8303,7 @@
         <v>TD: TD_P2_011 | [GIU NGUYEN] ID goc: AML_MT195_MND_01</v>
       </c>
     </row>
-    <row r="90" xml:space="preserve">
+    <row r="90" xml:space="preserve" outlineLevel="1">
       <c r="A90" s="5" t="str">
         <v>AML_MT195_MND_02</v>
       </c>
@@ -8378,7 +8381,7 @@
         <v>TD: TD_P2_011 | [GIU NGUYEN] ID goc: AML_MT195_MND_02</v>
       </c>
     </row>
-    <row r="91" xml:space="preserve">
+    <row r="91" xml:space="preserve" outlineLevel="1">
       <c r="A91" s="5" t="str">
         <v>AML_MT195_MND_03</v>
       </c>
@@ -8515,7 +8518,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" xml:space="preserve">
+    <row r="93" xml:space="preserve" outlineLevel="1">
       <c r="A93" s="5" t="str">
         <v>AML_MT196_MND_01</v>
       </c>
@@ -8652,7 +8655,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" xml:space="preserve">
+    <row r="95" xml:space="preserve" outlineLevel="1">
       <c r="A95" s="5" t="str">
         <v>AML_MT199_MND_01</v>
       </c>
@@ -8730,7 +8733,7 @@
         <v>TD: TD_P2_013 | [GIU NGUYEN] ID goc: AML_MT199_MND_01</v>
       </c>
     </row>
-    <row r="96" xml:space="preserve">
+    <row r="96" xml:space="preserve" outlineLevel="1">
       <c r="A96" s="5" t="str">
         <v>AML_MT199_MND_02</v>
       </c>
@@ -8867,7 +8870,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" xml:space="preserve">
+    <row r="98" xml:space="preserve" outlineLevel="1">
       <c r="A98" s="5" t="str">
         <v>AML_MT295_MND_01</v>
       </c>
@@ -8945,7 +8948,7 @@
         <v>TD: TD_P2_014 | [GIU NGUYEN] ID goc: AML_MT295_MND_01</v>
       </c>
     </row>
-    <row r="99" xml:space="preserve">
+    <row r="99" xml:space="preserve" outlineLevel="1">
       <c r="A99" s="5" t="str">
         <v>AML_MT295_MND_02</v>
       </c>
@@ -9023,7 +9026,7 @@
         <v>TD: TD_P2_014 | [GIU NGUYEN] ID goc: AML_MT295_MND_02</v>
       </c>
     </row>
-    <row r="100" xml:space="preserve">
+    <row r="100" xml:space="preserve" outlineLevel="1">
       <c r="A100" s="5" t="str">
         <v>AML_MT295_MND_03</v>
       </c>
@@ -9160,7 +9163,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" xml:space="preserve">
+    <row r="102" xml:space="preserve" outlineLevel="1">
       <c r="A102" s="5" t="str">
         <v>AML_MT296_MND_01</v>
       </c>
@@ -9238,7 +9241,7 @@
         <v>TD: TD_P2_015 | [GIU NGUYEN] ID goc: AML_MT296_MND_01</v>
       </c>
     </row>
-    <row r="103" xml:space="preserve">
+    <row r="103" xml:space="preserve" outlineLevel="1">
       <c r="A103" s="5" t="str">
         <v>AML_MT296_MND_02</v>
       </c>
@@ -9316,7 +9319,7 @@
         <v>TD: TD_P2_015 | [GIU NGUYEN] ID goc: AML_MT296_MND_02</v>
       </c>
     </row>
-    <row r="104" xml:space="preserve">
+    <row r="104" xml:space="preserve" outlineLevel="1">
       <c r="A104" s="5" t="str">
         <v>AML_MT296_MND_03</v>
       </c>
@@ -9453,7 +9456,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" xml:space="preserve">
+    <row r="106" xml:space="preserve" outlineLevel="1">
       <c r="A106" s="5" t="str">
         <v>AML_MT299_MND_01</v>
       </c>
@@ -9531,7 +9534,7 @@
         <v>TD: TD_P2_016 | [GIU NGUYEN] ID goc: AML_MT299_MND_01</v>
       </c>
     </row>
-    <row r="107" xml:space="preserve">
+    <row r="107" xml:space="preserve" outlineLevel="1">
       <c r="A107" s="5" t="str">
         <v>AML_MT299_MND_02</v>
       </c>
@@ -9668,7 +9671,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" xml:space="preserve">
+    <row r="109" xml:space="preserve" outlineLevel="1">
       <c r="A109" s="5" t="str">
         <v>AML_MT499_MND_01</v>
       </c>
@@ -9746,7 +9749,7 @@
         <v>TD: TD_P2_017 | [GIU NGUYEN] ID goc: AML_MT499_MND_01</v>
       </c>
     </row>
-    <row r="110" xml:space="preserve">
+    <row r="110" xml:space="preserve" outlineLevel="1">
       <c r="A110" s="5" t="str">
         <v>AML_MT499_MND_02</v>
       </c>
@@ -9883,7 +9886,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" xml:space="preserve">
+    <row r="112" xml:space="preserve" outlineLevel="1">
       <c r="A112" s="5" t="str">
         <v>AML_MT700_MND_01</v>
       </c>
@@ -9961,7 +9964,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_01</v>
       </c>
     </row>
-    <row r="113" xml:space="preserve">
+    <row r="113" xml:space="preserve" outlineLevel="1">
       <c r="A113" s="5" t="str">
         <v>AML_MT700_MND_02</v>
       </c>
@@ -10039,7 +10042,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_02</v>
       </c>
     </row>
-    <row r="114" xml:space="preserve">
+    <row r="114" xml:space="preserve" outlineLevel="1">
       <c r="A114" s="5" t="str">
         <v>AML_MT700_MND_03</v>
       </c>
@@ -10117,7 +10120,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_03</v>
       </c>
     </row>
-    <row r="115" xml:space="preserve">
+    <row r="115" xml:space="preserve" outlineLevel="1">
       <c r="A115" s="5" t="str">
         <v>AML_MT700_MND_04</v>
       </c>
@@ -10195,7 +10198,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_04</v>
       </c>
     </row>
-    <row r="116" xml:space="preserve">
+    <row r="116" xml:space="preserve" outlineLevel="1">
       <c r="A116" s="5" t="str">
         <v>AML_MT700_MND_05</v>
       </c>
@@ -10273,7 +10276,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_05</v>
       </c>
     </row>
-    <row r="117" xml:space="preserve">
+    <row r="117" xml:space="preserve" outlineLevel="1">
       <c r="A117" s="5" t="str">
         <v>AML_MT700_MND_06</v>
       </c>
@@ -10351,7 +10354,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_06</v>
       </c>
     </row>
-    <row r="118" xml:space="preserve">
+    <row r="118" xml:space="preserve" outlineLevel="1">
       <c r="A118" s="5" t="str">
         <v>AML_MT700_MND_07</v>
       </c>
@@ -10429,7 +10432,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_07</v>
       </c>
     </row>
-    <row r="119" xml:space="preserve">
+    <row r="119" xml:space="preserve" outlineLevel="1">
       <c r="A119" s="5" t="str">
         <v>AML_MT700_MND_08</v>
       </c>
@@ -10507,7 +10510,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_08</v>
       </c>
     </row>
-    <row r="120" xml:space="preserve">
+    <row r="120" xml:space="preserve" outlineLevel="1">
       <c r="A120" s="5" t="str">
         <v>AML_MT700_MND_09</v>
       </c>
@@ -10585,7 +10588,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_09</v>
       </c>
     </row>
-    <row r="121" xml:space="preserve">
+    <row r="121" xml:space="preserve" outlineLevel="1">
       <c r="A121" s="5" t="str">
         <v>AML_MT700_MND_10</v>
       </c>
@@ -10663,7 +10666,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_10</v>
       </c>
     </row>
-    <row r="122" xml:space="preserve">
+    <row r="122" xml:space="preserve" outlineLevel="1">
       <c r="A122" s="5" t="str">
         <v>AML_MT700_MND_11</v>
       </c>
@@ -10741,7 +10744,7 @@
         <v>TD: TD_P2_018 | [GIU NGUYEN] ID goc: AML_MT700_MND_11</v>
       </c>
     </row>
-    <row r="123" xml:space="preserve">
+    <row r="123" xml:space="preserve" outlineLevel="1">
       <c r="A123" s="5" t="str">
         <v>AML_MT700_MND_12</v>
       </c>
@@ -10878,7 +10881,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" xml:space="preserve">
+    <row r="125" xml:space="preserve" outlineLevel="1">
       <c r="A125" s="5" t="str">
         <v>AML_MT701_MND_01</v>
       </c>
@@ -10956,7 +10959,7 @@
         <v>TD: TD_P2_019 | [GIU NGUYEN] ID goc: AML_MT701_MND_01</v>
       </c>
     </row>
-    <row r="126" xml:space="preserve">
+    <row r="126" xml:space="preserve" outlineLevel="1">
       <c r="A126" s="5" t="str">
         <v>AML_MT701_MND_02</v>
       </c>
@@ -11093,7 +11096,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" xml:space="preserve">
+    <row r="128" xml:space="preserve" outlineLevel="1">
       <c r="A128" s="5" t="str">
         <v>AML_MT707_MND_01</v>
       </c>
@@ -11171,7 +11174,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_01</v>
       </c>
     </row>
-    <row r="129" xml:space="preserve">
+    <row r="129" xml:space="preserve" outlineLevel="1">
       <c r="A129" s="5" t="str">
         <v>AML_MT707_MND_02</v>
       </c>
@@ -11249,7 +11252,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_02</v>
       </c>
     </row>
-    <row r="130" xml:space="preserve">
+    <row r="130" xml:space="preserve" outlineLevel="1">
       <c r="A130" s="5" t="str">
         <v>AML_MT707_MND_03</v>
       </c>
@@ -11327,7 +11330,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_03</v>
       </c>
     </row>
-    <row r="131" xml:space="preserve">
+    <row r="131" xml:space="preserve" outlineLevel="1">
       <c r="A131" s="5" t="str">
         <v>AML_MT707_MND_04</v>
       </c>
@@ -11405,7 +11408,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_04</v>
       </c>
     </row>
-    <row r="132" xml:space="preserve">
+    <row r="132" xml:space="preserve" outlineLevel="1">
       <c r="A132" s="5" t="str">
         <v>AML_MT707_MND_05</v>
       </c>
@@ -11483,7 +11486,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_05</v>
       </c>
     </row>
-    <row r="133" xml:space="preserve">
+    <row r="133" xml:space="preserve" outlineLevel="1">
       <c r="A133" s="5" t="str">
         <v>AML_MT707_MND_06</v>
       </c>
@@ -11561,7 +11564,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_06</v>
       </c>
     </row>
-    <row r="134" xml:space="preserve">
+    <row r="134" xml:space="preserve" outlineLevel="1">
       <c r="A134" s="5" t="str">
         <v>AML_MT707_MND_07</v>
       </c>
@@ -11639,7 +11642,7 @@
         <v>TD: TD_P2_020 | [GIU NGUYEN] ID goc: AML_MT707_MND_07</v>
       </c>
     </row>
-    <row r="135" xml:space="preserve">
+    <row r="135" xml:space="preserve" outlineLevel="1">
       <c r="A135" s="5" t="str">
         <v>AML_MT707_MND_08</v>
       </c>
@@ -11776,7 +11779,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" xml:space="preserve">
+    <row r="137" xml:space="preserve" outlineLevel="1">
       <c r="A137" s="5" t="str">
         <v>AML_MT710_MND_01</v>
       </c>
@@ -11854,7 +11857,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_01</v>
       </c>
     </row>
-    <row r="138" xml:space="preserve">
+    <row r="138" xml:space="preserve" outlineLevel="1">
       <c r="A138" s="5" t="str">
         <v>AML_MT710_MND_02</v>
       </c>
@@ -11932,7 +11935,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_02</v>
       </c>
     </row>
-    <row r="139" xml:space="preserve">
+    <row r="139" xml:space="preserve" outlineLevel="1">
       <c r="A139" s="5" t="str">
         <v>AML_MT710_MND_03</v>
       </c>
@@ -12010,7 +12013,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_03</v>
       </c>
     </row>
-    <row r="140" xml:space="preserve">
+    <row r="140" xml:space="preserve" outlineLevel="1">
       <c r="A140" s="5" t="str">
         <v>AML_MT710_MND_04</v>
       </c>
@@ -12088,7 +12091,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_04</v>
       </c>
     </row>
-    <row r="141" xml:space="preserve">
+    <row r="141" xml:space="preserve" outlineLevel="1">
       <c r="A141" s="5" t="str">
         <v>AML_MT710_MND_05</v>
       </c>
@@ -12166,7 +12169,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_05</v>
       </c>
     </row>
-    <row r="142" xml:space="preserve">
+    <row r="142" xml:space="preserve" outlineLevel="1">
       <c r="A142" s="5" t="str">
         <v>AML_MT710_MND_06</v>
       </c>
@@ -12244,7 +12247,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_06</v>
       </c>
     </row>
-    <row r="143" xml:space="preserve">
+    <row r="143" xml:space="preserve" outlineLevel="1">
       <c r="A143" s="5" t="str">
         <v>AML_MT710_MND_07</v>
       </c>
@@ -12322,7 +12325,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_07</v>
       </c>
     </row>
-    <row r="144" xml:space="preserve">
+    <row r="144" xml:space="preserve" outlineLevel="1">
       <c r="A144" s="5" t="str">
         <v>AML_MT710_MND_08</v>
       </c>
@@ -12400,7 +12403,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_08</v>
       </c>
     </row>
-    <row r="145" xml:space="preserve">
+    <row r="145" xml:space="preserve" outlineLevel="1">
       <c r="A145" s="5" t="str">
         <v>AML_MT710_MND_09</v>
       </c>
@@ -12478,7 +12481,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_09</v>
       </c>
     </row>
-    <row r="146" xml:space="preserve">
+    <row r="146" xml:space="preserve" outlineLevel="1">
       <c r="A146" s="5" t="str">
         <v>AML_MT710_MND_10</v>
       </c>
@@ -12556,7 +12559,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_10</v>
       </c>
     </row>
-    <row r="147" xml:space="preserve">
+    <row r="147" xml:space="preserve" outlineLevel="1">
       <c r="A147" s="5" t="str">
         <v>AML_MT710_MND_11</v>
       </c>
@@ -12634,7 +12637,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_11</v>
       </c>
     </row>
-    <row r="148" xml:space="preserve">
+    <row r="148" xml:space="preserve" outlineLevel="1">
       <c r="A148" s="5" t="str">
         <v>AML_MT710_MND_12</v>
       </c>
@@ -12712,7 +12715,7 @@
         <v>TD: TD_P2_021 | [GIU NGUYEN] ID goc: AML_MT710_MND_12</v>
       </c>
     </row>
-    <row r="149" xml:space="preserve">
+    <row r="149" xml:space="preserve" outlineLevel="1">
       <c r="A149" s="5" t="str">
         <v>AML_MT710_MND_13</v>
       </c>
@@ -12849,7 +12852,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" xml:space="preserve">
+    <row r="151" xml:space="preserve" outlineLevel="1">
       <c r="A151" s="5" t="str">
         <v>AML_MT711_MND_01</v>
       </c>
@@ -12927,7 +12930,7 @@
         <v>TD: TD_P2_022 | [GIU NGUYEN] ID goc: AML_MT711_MND_01</v>
       </c>
     </row>
-    <row r="152" xml:space="preserve">
+    <row r="152" xml:space="preserve" outlineLevel="1">
       <c r="A152" s="5" t="str">
         <v>AML_MT711_MND_02</v>
       </c>
@@ -13005,7 +13008,7 @@
         <v>TD: TD_P2_022 | [GIU NGUYEN] ID goc: AML_MT711_MND_02</v>
       </c>
     </row>
-    <row r="153" xml:space="preserve">
+    <row r="153" xml:space="preserve" outlineLevel="1">
       <c r="A153" s="5" t="str">
         <v>AML_MT711_MND_03</v>
       </c>
@@ -13142,7 +13145,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" xml:space="preserve">
+    <row r="155" xml:space="preserve" outlineLevel="1">
       <c r="A155" s="5" t="str">
         <v>AML_MT720_MND_01</v>
       </c>
@@ -13220,7 +13223,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_01</v>
       </c>
     </row>
-    <row r="156" xml:space="preserve">
+    <row r="156" xml:space="preserve" outlineLevel="1">
       <c r="A156" s="5" t="str">
         <v>AML_MT720_MND_02</v>
       </c>
@@ -13298,7 +13301,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_02</v>
       </c>
     </row>
-    <row r="157" xml:space="preserve">
+    <row r="157" xml:space="preserve" outlineLevel="1">
       <c r="A157" s="5" t="str">
         <v>AML_MT720_MND_03</v>
       </c>
@@ -13376,7 +13379,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_03</v>
       </c>
     </row>
-    <row r="158" xml:space="preserve">
+    <row r="158" xml:space="preserve" outlineLevel="1">
       <c r="A158" s="5" t="str">
         <v>AML_MT720_MND_04</v>
       </c>
@@ -13454,7 +13457,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_04</v>
       </c>
     </row>
-    <row r="159" xml:space="preserve">
+    <row r="159" xml:space="preserve" outlineLevel="1">
       <c r="A159" s="5" t="str">
         <v>AML_MT720_MND_05</v>
       </c>
@@ -13532,7 +13535,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_05</v>
       </c>
     </row>
-    <row r="160" xml:space="preserve">
+    <row r="160" xml:space="preserve" outlineLevel="1">
       <c r="A160" s="5" t="str">
         <v>AML_MT720_MND_06</v>
       </c>
@@ -13610,7 +13613,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_06</v>
       </c>
     </row>
-    <row r="161" xml:space="preserve">
+    <row r="161" xml:space="preserve" outlineLevel="1">
       <c r="A161" s="5" t="str">
         <v>AML_MT720_MND_07</v>
       </c>
@@ -13688,7 +13691,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_07</v>
       </c>
     </row>
-    <row r="162" xml:space="preserve">
+    <row r="162" xml:space="preserve" outlineLevel="1">
       <c r="A162" s="5" t="str">
         <v>AML_MT720_MND_08</v>
       </c>
@@ -13766,7 +13769,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_08</v>
       </c>
     </row>
-    <row r="163" xml:space="preserve">
+    <row r="163" xml:space="preserve" outlineLevel="1">
       <c r="A163" s="5" t="str">
         <v>AML_MT720_MND_09</v>
       </c>
@@ -13844,7 +13847,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_09</v>
       </c>
     </row>
-    <row r="164" xml:space="preserve">
+    <row r="164" xml:space="preserve" outlineLevel="1">
       <c r="A164" s="5" t="str">
         <v>AML_MT720_MND_10</v>
       </c>
@@ -13922,7 +13925,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_10</v>
       </c>
     </row>
-    <row r="165" xml:space="preserve">
+    <row r="165" xml:space="preserve" outlineLevel="1">
       <c r="A165" s="5" t="str">
         <v>AML_MT720_MND_11</v>
       </c>
@@ -14000,7 +14003,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_11</v>
       </c>
     </row>
-    <row r="166" xml:space="preserve">
+    <row r="166" xml:space="preserve" outlineLevel="1">
       <c r="A166" s="5" t="str">
         <v>AML_MT720_MND_12</v>
       </c>
@@ -14078,7 +14081,7 @@
         <v>TD: TD_P2_023 | [GIU NGUYEN] ID goc: AML_MT720_MND_12</v>
       </c>
     </row>
-    <row r="167" xml:space="preserve">
+    <row r="167" xml:space="preserve" outlineLevel="1">
       <c r="A167" s="5" t="str">
         <v>AML_MT720_MND_13</v>
       </c>
@@ -14215,7 +14218,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" xml:space="preserve">
+    <row r="169" xml:space="preserve" outlineLevel="1">
       <c r="A169" s="5" t="str">
         <v>AML_MT740_MND_01</v>
       </c>
@@ -14293,7 +14296,7 @@
         <v>TD: TD_P2_024 | [GIU NGUYEN] ID goc: AML_MT740_MND_01</v>
       </c>
     </row>
-    <row r="170" xml:space="preserve">
+    <row r="170" xml:space="preserve" outlineLevel="1">
       <c r="A170" s="5" t="str">
         <v>AML_MT740_MND_02</v>
       </c>
@@ -14371,7 +14374,7 @@
         <v>TD: TD_P2_024 | [GIU NGUYEN] ID goc: AML_MT740_MND_02</v>
       </c>
     </row>
-    <row r="171" xml:space="preserve">
+    <row r="171" xml:space="preserve" outlineLevel="1">
       <c r="A171" s="5" t="str">
         <v>AML_MT740_MND_03</v>
       </c>
@@ -14449,7 +14452,7 @@
         <v>TD: TD_P2_024 | [GIU NGUYEN] ID goc: AML_MT740_MND_03</v>
       </c>
     </row>
-    <row r="172" xml:space="preserve">
+    <row r="172" xml:space="preserve" outlineLevel="1">
       <c r="A172" s="5" t="str">
         <v>AML_MT740_MND_04</v>
       </c>
@@ -14527,7 +14530,7 @@
         <v>TD: TD_P2_024 | [GIU NGUYEN] ID goc: AML_MT740_MND_04</v>
       </c>
     </row>
-    <row r="173" xml:space="preserve">
+    <row r="173" xml:space="preserve" outlineLevel="1">
       <c r="A173" s="5" t="str">
         <v>AML_MT740_MND_05</v>
       </c>
@@ -14664,7 +14667,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" xml:space="preserve">
+    <row r="175" xml:space="preserve" outlineLevel="1">
       <c r="A175" s="5" t="str">
         <v>AML_MT742_MND_01</v>
       </c>
@@ -14742,7 +14745,7 @@
         <v>TD: TD_P2_025 | [GIU NGUYEN] ID goc: AML_MT742_MND_01</v>
       </c>
     </row>
-    <row r="176" xml:space="preserve">
+    <row r="176" xml:space="preserve" outlineLevel="1">
       <c r="A176" s="5" t="str">
         <v>AML_MT742_MND_02</v>
       </c>
@@ -14820,7 +14823,7 @@
         <v>TD: TD_P2_025 | [GIU NGUYEN] ID goc: AML_MT742_MND_02</v>
       </c>
     </row>
-    <row r="177" xml:space="preserve">
+    <row r="177" xml:space="preserve" outlineLevel="1">
       <c r="A177" s="5" t="str">
         <v>AML_MT742_MND_03</v>
       </c>
@@ -14898,7 +14901,7 @@
         <v>TD: TD_P2_025 | [GIU NGUYEN] ID goc: AML_MT742_MND_03</v>
       </c>
     </row>
-    <row r="178" xml:space="preserve">
+    <row r="178" xml:space="preserve" outlineLevel="1">
       <c r="A178" s="5" t="str">
         <v>AML_MT742_MND_04</v>
       </c>
@@ -14976,7 +14979,7 @@
         <v>TD: TD_P2_025 | [GIU NGUYEN] ID goc: AML_MT742_MND_04</v>
       </c>
     </row>
-    <row r="179" xml:space="preserve">
+    <row r="179" xml:space="preserve" outlineLevel="1">
       <c r="A179" s="5" t="str">
         <v>AML_MT742_MND_05</v>
       </c>
@@ -15054,7 +15057,7 @@
         <v>TD: TD_P2_025 | [GIU NGUYEN] ID goc: AML_MT742_MND_05</v>
       </c>
     </row>
-    <row r="180" xml:space="preserve">
+    <row r="180" xml:space="preserve" outlineLevel="1">
       <c r="A180" s="5" t="str">
         <v>AML_MT742_MND_06</v>
       </c>
@@ -15132,7 +15135,7 @@
         <v>TD: TD_P2_025 | [GIU NGUYEN] ID goc: AML_MT742_MND_06</v>
       </c>
     </row>
-    <row r="181" xml:space="preserve">
+    <row r="181" xml:space="preserve" outlineLevel="1">
       <c r="A181" s="5" t="str">
         <v>AML_MT742_MND_07</v>
       </c>
@@ -15269,7 +15272,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" xml:space="preserve">
+    <row r="183" xml:space="preserve" outlineLevel="1">
       <c r="A183" s="5" t="str">
         <v>AML_MT747_MND_01</v>
       </c>
@@ -15347,7 +15350,7 @@
         <v>TD: TD_P2_026 | [GIU NGUYEN] ID goc: AML_MT747_MND_01</v>
       </c>
     </row>
-    <row r="184" xml:space="preserve">
+    <row r="184" xml:space="preserve" outlineLevel="1">
       <c r="A184" s="5" t="str">
         <v>AML_MT747_MND_02</v>
       </c>
@@ -15484,7 +15487,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" xml:space="preserve">
+    <row r="186" xml:space="preserve" outlineLevel="1">
       <c r="A186" s="5" t="str">
         <v>AML_MT760_MND_01</v>
       </c>
@@ -15562,7 +15565,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_01</v>
       </c>
     </row>
-    <row r="187" xml:space="preserve">
+    <row r="187" xml:space="preserve" outlineLevel="1">
       <c r="A187" s="5" t="str">
         <v>AML_MT760_MND_02</v>
       </c>
@@ -15640,7 +15643,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_02</v>
       </c>
     </row>
-    <row r="188" xml:space="preserve">
+    <row r="188" xml:space="preserve" outlineLevel="1">
       <c r="A188" s="5" t="str">
         <v>AML_MT760_MND_03</v>
       </c>
@@ -15718,7 +15721,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_03</v>
       </c>
     </row>
-    <row r="189" xml:space="preserve">
+    <row r="189" xml:space="preserve" outlineLevel="1">
       <c r="A189" s="5" t="str">
         <v>AML_MT760_MND_04</v>
       </c>
@@ -15796,7 +15799,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_04</v>
       </c>
     </row>
-    <row r="190" xml:space="preserve">
+    <row r="190" xml:space="preserve" outlineLevel="1">
       <c r="A190" s="5" t="str">
         <v>AML_MT760_MND_05</v>
       </c>
@@ -15874,7 +15877,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_05</v>
       </c>
     </row>
-    <row r="191" xml:space="preserve">
+    <row r="191" xml:space="preserve" outlineLevel="1">
       <c r="A191" s="5" t="str">
         <v>AML_MT760_MND_06</v>
       </c>
@@ -15952,7 +15955,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_06</v>
       </c>
     </row>
-    <row r="192" xml:space="preserve">
+    <row r="192" xml:space="preserve" outlineLevel="1">
       <c r="A192" s="5" t="str">
         <v>AML_MT760_MND_07</v>
       </c>
@@ -16030,7 +16033,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_07</v>
       </c>
     </row>
-    <row r="193" xml:space="preserve">
+    <row r="193" xml:space="preserve" outlineLevel="1">
       <c r="A193" s="5" t="str">
         <v>AML_MT760_MND_08</v>
       </c>
@@ -16108,7 +16111,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_08</v>
       </c>
     </row>
-    <row r="194" xml:space="preserve">
+    <row r="194" xml:space="preserve" outlineLevel="1">
       <c r="A194" s="5" t="str">
         <v>AML_MT760_MND_09</v>
       </c>
@@ -16186,7 +16189,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_09</v>
       </c>
     </row>
-    <row r="195" xml:space="preserve">
+    <row r="195" xml:space="preserve" outlineLevel="1">
       <c r="A195" s="5" t="str">
         <v>AML_MT760_MND_10</v>
       </c>
@@ -16264,7 +16267,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_10</v>
       </c>
     </row>
-    <row r="196" xml:space="preserve">
+    <row r="196" xml:space="preserve" outlineLevel="1">
       <c r="A196" s="5" t="str">
         <v>AML_MT760_MND_11</v>
       </c>
@@ -16342,7 +16345,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_11</v>
       </c>
     </row>
-    <row r="197" xml:space="preserve">
+    <row r="197" xml:space="preserve" outlineLevel="1">
       <c r="A197" s="5" t="str">
         <v>AML_MT760_MND_12</v>
       </c>
@@ -16420,7 +16423,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_12</v>
       </c>
     </row>
-    <row r="198" xml:space="preserve">
+    <row r="198" xml:space="preserve" outlineLevel="1">
       <c r="A198" s="5" t="str">
         <v>AML_MT760_MND_13</v>
       </c>
@@ -16498,7 +16501,7 @@
         <v>TD: TD_P2_027 | [GIU NGUYEN] ID goc: AML_MT760_MND_13</v>
       </c>
     </row>
-    <row r="199" xml:space="preserve">
+    <row r="199" xml:space="preserve" outlineLevel="1">
       <c r="A199" s="5" t="str">
         <v>AML_MT760_MND_14</v>
       </c>
@@ -16635,7 +16638,7 @@
         <v/>
       </c>
     </row>
-    <row r="201" xml:space="preserve">
+    <row r="201" xml:space="preserve" outlineLevel="1">
       <c r="A201" s="5" t="str">
         <v>AML_MT767_MND_01</v>
       </c>
@@ -16713,7 +16716,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_01</v>
       </c>
     </row>
-    <row r="202" xml:space="preserve">
+    <row r="202" xml:space="preserve" outlineLevel="1">
       <c r="A202" s="5" t="str">
         <v>AML_MT767_MND_02</v>
       </c>
@@ -16791,7 +16794,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_02</v>
       </c>
     </row>
-    <row r="203" xml:space="preserve">
+    <row r="203" xml:space="preserve" outlineLevel="1">
       <c r="A203" s="5" t="str">
         <v>AML_MT767_MND_03</v>
       </c>
@@ -16869,7 +16872,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_03</v>
       </c>
     </row>
-    <row r="204" xml:space="preserve">
+    <row r="204" xml:space="preserve" outlineLevel="1">
       <c r="A204" s="5" t="str">
         <v>AML_MT767_MND_04</v>
       </c>
@@ -16947,7 +16950,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_04</v>
       </c>
     </row>
-    <row r="205" xml:space="preserve">
+    <row r="205" xml:space="preserve" outlineLevel="1">
       <c r="A205" s="5" t="str">
         <v>AML_MT767_MND_05</v>
       </c>
@@ -17025,7 +17028,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_05</v>
       </c>
     </row>
-    <row r="206" xml:space="preserve">
+    <row r="206" xml:space="preserve" outlineLevel="1">
       <c r="A206" s="5" t="str">
         <v>AML_MT767_MND_06</v>
       </c>
@@ -17103,7 +17106,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_06</v>
       </c>
     </row>
-    <row r="207" xml:space="preserve">
+    <row r="207" xml:space="preserve" outlineLevel="1">
       <c r="A207" s="5" t="str">
         <v>AML_MT767_MND_07</v>
       </c>
@@ -17181,7 +17184,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_07</v>
       </c>
     </row>
-    <row r="208" xml:space="preserve">
+    <row r="208" xml:space="preserve" outlineLevel="1">
       <c r="A208" s="5" t="str">
         <v>AML_MT767_MND_08</v>
       </c>
@@ -17259,7 +17262,7 @@
         <v>TD: TD_P2_028 | [GIU NGUYEN] ID goc: AML_MT767_MND_08</v>
       </c>
     </row>
-    <row r="209" xml:space="preserve">
+    <row r="209" xml:space="preserve" outlineLevel="1">
       <c r="A209" s="5" t="str">
         <v>AML_MT767_MND_09</v>
       </c>
@@ -17396,7 +17399,7 @@
         <v/>
       </c>
     </row>
-    <row r="211" xml:space="preserve">
+    <row r="211" xml:space="preserve" outlineLevel="1">
       <c r="A211" s="5" t="str">
         <v>AML_MT799_MND_01</v>
       </c>
@@ -17474,7 +17477,7 @@
         <v>TD: TD_P2_029 | [GIU NGUYEN] ID goc: AML_MT799_MND_01</v>
       </c>
     </row>
-    <row r="212" xml:space="preserve">
+    <row r="212" xml:space="preserve" outlineLevel="1">
       <c r="A212" s="5" t="str">
         <v>AML_MT799_MND_02</v>
       </c>
@@ -17611,7 +17614,7 @@
         <v/>
       </c>
     </row>
-    <row r="214" xml:space="preserve">
+    <row r="214" xml:space="preserve" outlineLevel="1">
       <c r="A214" s="5" t="str">
         <v>AML_MT999_MND_01</v>
       </c>
@@ -17689,7 +17692,7 @@
         <v>TD: TD_P2_030 | [GIU NGUYEN] ID goc: AML_MT999_MND_01</v>
       </c>
     </row>
-    <row r="215" xml:space="preserve">
+    <row r="215" xml:space="preserve" outlineLevel="1">
       <c r="A215" s="5" t="str">
         <v>AML_MT999_MND_02</v>
       </c>
@@ -17826,7 +17829,7 @@
         <v/>
       </c>
     </row>
-    <row r="217" xml:space="preserve">
+    <row r="217" xml:space="preserve" outlineLevel="1">
       <c r="A217" s="5" t="str">
         <v>AML_PACS009_MND_01</v>
       </c>
@@ -17902,7 +17905,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_01</v>
       </c>
     </row>
-    <row r="218" xml:space="preserve">
+    <row r="218" xml:space="preserve" outlineLevel="1">
       <c r="A218" s="5" t="str">
         <v>AML_PACS009_MND_02</v>
       </c>
@@ -17978,7 +17981,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_02</v>
       </c>
     </row>
-    <row r="219" xml:space="preserve">
+    <row r="219" xml:space="preserve" outlineLevel="1">
       <c r="A219" s="5" t="str">
         <v>AML_PACS009_MND_05</v>
       </c>
@@ -18054,7 +18057,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_05</v>
       </c>
     </row>
-    <row r="220" xml:space="preserve">
+    <row r="220" xml:space="preserve" outlineLevel="1">
       <c r="A220" s="5" t="str">
         <v>AML_PACS009_MND_06</v>
       </c>
@@ -18130,7 +18133,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_06</v>
       </c>
     </row>
-    <row r="221" xml:space="preserve">
+    <row r="221" xml:space="preserve" outlineLevel="1">
       <c r="A221" s="5" t="str">
         <v>AML_PACS009_MND_07</v>
       </c>
@@ -18206,7 +18209,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_07</v>
       </c>
     </row>
-    <row r="222" xml:space="preserve">
+    <row r="222" xml:space="preserve" outlineLevel="1">
       <c r="A222" s="5" t="str">
         <v>AML_PACS009_MND_08</v>
       </c>
@@ -18282,7 +18285,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_08</v>
       </c>
     </row>
-    <row r="223" xml:space="preserve">
+    <row r="223" xml:space="preserve" outlineLevel="1">
       <c r="A223" s="5" t="str">
         <v>AML_PACS009_MND_09</v>
       </c>
@@ -18358,7 +18361,7 @@
         <v>TD: TD_P2_033 | [GIU NGUYEN] ID goc: AML_PACS009_MND_09</v>
       </c>
     </row>
-    <row r="224" xml:space="preserve">
+    <row r="224" xml:space="preserve" outlineLevel="1">
       <c r="A224" s="5" t="str">
         <v>AML_PACS009_MND_10</v>
       </c>
@@ -18493,7 +18496,7 @@
         <v/>
       </c>
     </row>
-    <row r="226" xml:space="preserve">
+    <row r="226" xml:space="preserve" outlineLevel="1">
       <c r="A226" s="5" t="str">
         <v>AML_PACS004_MND_01</v>
       </c>
@@ -18569,7 +18572,7 @@
         <v>TD: TD_P2_034 | [GIU NGUYEN] ID goc: AML_PACS004_MND_01</v>
       </c>
     </row>
-    <row r="227" xml:space="preserve">
+    <row r="227" xml:space="preserve" outlineLevel="1">
       <c r="A227" s="5" t="str">
         <v>AML_PACS004_MND_02</v>
       </c>
@@ -18645,7 +18648,7 @@
         <v>TD: TD_P2_034 | [GIU NGUYEN] ID goc: AML_PACS004_MND_02</v>
       </c>
     </row>
-    <row r="228" xml:space="preserve">
+    <row r="228" xml:space="preserve" outlineLevel="1">
       <c r="A228" s="5" t="str">
         <v>AML_PACS004_MND_03</v>
       </c>
@@ -18721,7 +18724,7 @@
         <v>TD: TD_P2_034 | [GIU NGUYEN] ID goc: AML_PACS004_MND_03</v>
       </c>
     </row>
-    <row r="229" xml:space="preserve">
+    <row r="229" xml:space="preserve" outlineLevel="1">
       <c r="A229" s="5" t="str">
         <v>AML_PACS004_MND_04</v>
       </c>
@@ -18856,7 +18859,7 @@
         <v/>
       </c>
     </row>
-    <row r="231" xml:space="preserve">
+    <row r="231" xml:space="preserve" outlineLevel="1">
       <c r="A231" s="5" t="str">
         <v>AML_PACS008_MND_01</v>
       </c>
@@ -18932,7 +18935,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_01</v>
       </c>
     </row>
-    <row r="232" xml:space="preserve">
+    <row r="232" xml:space="preserve" outlineLevel="1">
       <c r="A232" s="5" t="str">
         <v>AML_PACS008_MND_02</v>
       </c>
@@ -19008,7 +19011,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_02</v>
       </c>
     </row>
-    <row r="233" xml:space="preserve">
+    <row r="233" xml:space="preserve" outlineLevel="1">
       <c r="A233" s="5" t="str">
         <v>AML_PACS008_MND_03</v>
       </c>
@@ -19084,7 +19087,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_03</v>
       </c>
     </row>
-    <row r="234" xml:space="preserve">
+    <row r="234" xml:space="preserve" outlineLevel="1">
       <c r="A234" s="5" t="str">
         <v>AML_PACS008_MND_04</v>
       </c>
@@ -19160,7 +19163,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_04</v>
       </c>
     </row>
-    <row r="235" xml:space="preserve">
+    <row r="235" xml:space="preserve" outlineLevel="1">
       <c r="A235" s="5" t="str">
         <v>AML_PACS008_MND_05</v>
       </c>
@@ -19236,7 +19239,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_05</v>
       </c>
     </row>
-    <row r="236" xml:space="preserve">
+    <row r="236" xml:space="preserve" outlineLevel="1">
       <c r="A236" s="5" t="str">
         <v>AML_PACS008_MND_06</v>
       </c>
@@ -19312,7 +19315,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_06</v>
       </c>
     </row>
-    <row r="237" xml:space="preserve">
+    <row r="237" xml:space="preserve" outlineLevel="1">
       <c r="A237" s="5" t="str">
         <v>AML_PACS008_MND_07</v>
       </c>
@@ -19388,7 +19391,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_07</v>
       </c>
     </row>
-    <row r="238" xml:space="preserve">
+    <row r="238" xml:space="preserve" outlineLevel="1">
       <c r="A238" s="5" t="str">
         <v>AML_PACS008_MND_08</v>
       </c>
@@ -19464,7 +19467,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_08</v>
       </c>
     </row>
-    <row r="239" xml:space="preserve">
+    <row r="239" xml:space="preserve" outlineLevel="1">
       <c r="A239" s="5" t="str">
         <v>AML_PACS008_MND_09</v>
       </c>
@@ -19540,7 +19543,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_09</v>
       </c>
     </row>
-    <row r="240" xml:space="preserve">
+    <row r="240" xml:space="preserve" outlineLevel="1">
       <c r="A240" s="5" t="str">
         <v>AML_PACS008_MND_10</v>
       </c>
@@ -19616,7 +19619,7 @@
         <v>TD: TD_P2_035 | [GIU NGUYEN] ID goc: AML_PACS008_MND_10</v>
       </c>
     </row>
-    <row r="241" xml:space="preserve">
+    <row r="241" xml:space="preserve" outlineLevel="1">
       <c r="A241" s="5" t="str">
         <v>AML_PACS008_MND_11</v>
       </c>
@@ -19751,7 +19754,7 @@
         <v/>
       </c>
     </row>
-    <row r="243" xml:space="preserve">
+    <row r="243" xml:space="preserve" outlineLevel="1">
       <c r="A243" s="5" t="str">
         <v>AML_CAM110_MND_01</v>
       </c>
@@ -19827,7 +19830,7 @@
         <v>TD: TD_P2_036 | [GIU NGUYEN] ID goc: AML_CAM110_MND_01</v>
       </c>
     </row>
-    <row r="244" xml:space="preserve">
+    <row r="244" xml:space="preserve" outlineLevel="1">
       <c r="A244" s="5" t="str">
         <v>AML_CAM110_MND_02</v>
       </c>
@@ -19903,7 +19906,7 @@
         <v>TD: TD_P2_036 | [GIU NGUYEN] ID goc: AML_CAM110_MND_02</v>
       </c>
     </row>
-    <row r="245" xml:space="preserve">
+    <row r="245" xml:space="preserve" outlineLevel="1">
       <c r="A245" s="5" t="str">
         <v>AML_CAM110_MND_03</v>
       </c>
@@ -19979,7 +19982,7 @@
         <v>TD: TD_P2_036 | [GIU NGUYEN] ID goc: AML_CAM110_MND_03</v>
       </c>
     </row>
-    <row r="246" xml:space="preserve">
+    <row r="246" xml:space="preserve" outlineLevel="1">
       <c r="A246" s="5" t="str">
         <v>AML_CAM110_MND_04</v>
       </c>
@@ -20055,7 +20058,7 @@
         <v>TD: TD_P2_036 | [GIU NGUYEN] ID goc: AML_CAM110_MND_04</v>
       </c>
     </row>
-    <row r="247" xml:space="preserve">
+    <row r="247" xml:space="preserve" outlineLevel="1">
       <c r="A247" s="5" t="str">
         <v>AML_CAM110_MND_05</v>
       </c>
@@ -20131,7 +20134,7 @@
         <v>TD: TD_P2_036 | [GIU NGUYEN] ID goc: AML_CAM110_MND_05</v>
       </c>
     </row>
-    <row r="248" xml:space="preserve">
+    <row r="248" xml:space="preserve" outlineLevel="1">
       <c r="A248" s="5" t="str">
         <v>AML_CAM110_MND_06</v>
       </c>
@@ -20266,7 +20269,7 @@
         <v/>
       </c>
     </row>
-    <row r="250" xml:space="preserve">
+    <row r="250" xml:space="preserve" outlineLevel="1">
       <c r="A250" s="5" t="str">
         <v>AML_CAM111_MND_01</v>
       </c>
@@ -20342,7 +20345,7 @@
         <v>TD: TD_P2_037 | [GIU NGUYEN] ID goc: AML_CAM111_MND_01</v>
       </c>
     </row>
-    <row r="251" xml:space="preserve">
+    <row r="251" xml:space="preserve" outlineLevel="1">
       <c r="A251" s="5" t="str">
         <v>AML_CAM111_MND_02</v>
       </c>
@@ -20418,7 +20421,7 @@
         <v>TD: TD_P2_037 | [GIU NGUYEN] ID goc: AML_CAM111_MND_02</v>
       </c>
     </row>
-    <row r="252" xml:space="preserve">
+    <row r="252" xml:space="preserve" outlineLevel="1">
       <c r="A252" s="5" t="str">
         <v>AML_CAM111_MND_03</v>
       </c>
@@ -20494,7 +20497,7 @@
         <v>TD: TD_P2_037 | [GIU NGUYEN] ID goc: AML_CAM111_MND_03</v>
       </c>
     </row>
-    <row r="253" xml:space="preserve">
+    <row r="253" xml:space="preserve" outlineLevel="1">
       <c r="A253" s="5" t="str">
         <v>AML_CAM111_MND_04</v>
       </c>
@@ -20570,7 +20573,7 @@
         <v>TD: TD_P2_037 | [GIU NGUYEN] ID goc: AML_CAM111_MND_04</v>
       </c>
     </row>
-    <row r="254" xml:space="preserve">
+    <row r="254" xml:space="preserve" outlineLevel="1">
       <c r="A254" s="5" t="str">
         <v>AML_CAM111_MND_05</v>
       </c>
@@ -20646,7 +20649,7 @@
         <v>TD: TD_P2_037 | [GIU NGUYEN] ID goc: AML_CAM111_MND_05</v>
       </c>
     </row>
-    <row r="255" xml:space="preserve">
+    <row r="255" xml:space="preserve" outlineLevel="1">
       <c r="A255" s="5" t="str">
         <v>AML_CAM111_MND_06</v>
       </c>
@@ -20781,7 +20784,7 @@
         <v/>
       </c>
     </row>
-    <row r="257" xml:space="preserve">
+    <row r="257" xml:space="preserve" outlineLevel="1">
       <c r="A257" s="5" t="str">
         <v>AML_MSB001_MND_02</v>
       </c>
@@ -20857,7 +20860,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_02</v>
       </c>
     </row>
-    <row r="258" xml:space="preserve">
+    <row r="258" xml:space="preserve" outlineLevel="1">
       <c r="A258" s="5" t="str">
         <v>AML_MSB001_MND_03</v>
       </c>
@@ -20933,7 +20936,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_03</v>
       </c>
     </row>
-    <row r="259" xml:space="preserve">
+    <row r="259" xml:space="preserve" outlineLevel="1">
       <c r="A259" s="5" t="str">
         <v>AML_MSB001_MND_04</v>
       </c>
@@ -21009,7 +21012,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_04</v>
       </c>
     </row>
-    <row r="260" xml:space="preserve">
+    <row r="260" xml:space="preserve" outlineLevel="1">
       <c r="A260" s="5" t="str">
         <v>AML_MSB001_MND_05</v>
       </c>
@@ -21085,7 +21088,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_05</v>
       </c>
     </row>
-    <row r="261" xml:space="preserve">
+    <row r="261" xml:space="preserve" outlineLevel="1">
       <c r="A261" s="5" t="str">
         <v>AML_MSB001_MND_06</v>
       </c>
@@ -21161,7 +21164,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_06</v>
       </c>
     </row>
-    <row r="262" xml:space="preserve">
+    <row r="262" xml:space="preserve" outlineLevel="1">
       <c r="A262" s="5" t="str">
         <v>AML_MSB001_MND_07</v>
       </c>
@@ -21237,7 +21240,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_07</v>
       </c>
     </row>
-    <row r="263" xml:space="preserve">
+    <row r="263" xml:space="preserve" outlineLevel="1">
       <c r="A263" s="5" t="str">
         <v>AML_MSB001_MND_08</v>
       </c>
@@ -21313,7 +21316,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_08</v>
       </c>
     </row>
-    <row r="264" xml:space="preserve">
+    <row r="264" xml:space="preserve" outlineLevel="1">
       <c r="A264" s="5" t="str">
         <v>AML_MSB001_MND_09</v>
       </c>
@@ -21389,7 +21392,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_09</v>
       </c>
     </row>
-    <row r="265" xml:space="preserve">
+    <row r="265" xml:space="preserve" outlineLevel="1">
       <c r="A265" s="5" t="str">
         <v>AML_MSB001_MND_10</v>
       </c>
@@ -21465,7 +21468,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_10</v>
       </c>
     </row>
-    <row r="266" xml:space="preserve">
+    <row r="266" xml:space="preserve" outlineLevel="1">
       <c r="A266" s="5" t="str">
         <v>AML_MSB001_MND_11</v>
       </c>
@@ -21541,7 +21544,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_11</v>
       </c>
     </row>
-    <row r="267" xml:space="preserve">
+    <row r="267" xml:space="preserve" outlineLevel="1">
       <c r="A267" s="5" t="str">
         <v>AML_MSB001_MND_12</v>
       </c>
@@ -21617,7 +21620,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_12</v>
       </c>
     </row>
-    <row r="268" xml:space="preserve">
+    <row r="268" xml:space="preserve" outlineLevel="1">
       <c r="A268" s="5" t="str">
         <v>AML_MSB001_MND_13</v>
       </c>
@@ -21693,7 +21696,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_13</v>
       </c>
     </row>
-    <row r="269" xml:space="preserve">
+    <row r="269" xml:space="preserve" outlineLevel="1">
       <c r="A269" s="5" t="str">
         <v>AML_MSB001_MND_14</v>
       </c>
@@ -21769,7 +21772,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_14</v>
       </c>
     </row>
-    <row r="270" xml:space="preserve">
+    <row r="270" xml:space="preserve" outlineLevel="1">
       <c r="A270" s="5" t="str">
         <v>AML_MSB001_MND_15</v>
       </c>
@@ -21845,7 +21848,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_15</v>
       </c>
     </row>
-    <row r="271" xml:space="preserve">
+    <row r="271" xml:space="preserve" outlineLevel="1">
       <c r="A271" s="5" t="str">
         <v>AML_MSB001_MND_16</v>
       </c>
@@ -21921,7 +21924,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_16</v>
       </c>
     </row>
-    <row r="272" xml:space="preserve">
+    <row r="272" xml:space="preserve" outlineLevel="1">
       <c r="A272" s="5" t="str">
         <v>AML_MSB001_MND_17</v>
       </c>
@@ -21997,7 +22000,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_17</v>
       </c>
     </row>
-    <row r="273" xml:space="preserve">
+    <row r="273" xml:space="preserve" outlineLevel="1">
       <c r="A273" s="5" t="str">
         <v>AML_MSB001_MND_18</v>
       </c>
@@ -22073,7 +22076,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_18</v>
       </c>
     </row>
-    <row r="274" xml:space="preserve">
+    <row r="274" xml:space="preserve" outlineLevel="1">
       <c r="A274" s="5" t="str">
         <v>AML_MSB001_MND_19</v>
       </c>
@@ -22149,7 +22152,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_19</v>
       </c>
     </row>
-    <row r="275" xml:space="preserve">
+    <row r="275" xml:space="preserve" outlineLevel="1">
       <c r="A275" s="5" t="str">
         <v>AML_MSB001_MND_20</v>
       </c>
@@ -22225,7 +22228,7 @@
         <v>TD: TD_P2_040 | [GIU NGUYEN] ID goc: AML_MSB001_MND_20</v>
       </c>
     </row>
-    <row r="276" xml:space="preserve">
+    <row r="276" xml:space="preserve" outlineLevel="1">
       <c r="A276" s="5" t="str">
         <v>AML_MSB001_MND_21</v>
       </c>
@@ -22360,7 +22363,7 @@
         <v/>
       </c>
     </row>
-    <row r="278" xml:space="preserve">
+    <row r="278" xml:space="preserve" outlineLevel="1">
       <c r="A278" s="5" t="str">
         <v>AML_MSB002_MND_02</v>
       </c>
@@ -22436,7 +22439,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_02</v>
       </c>
     </row>
-    <row r="279" xml:space="preserve">
+    <row r="279" xml:space="preserve" outlineLevel="1">
       <c r="A279" s="5" t="str">
         <v>AML_MSB002_MND_03</v>
       </c>
@@ -22512,7 +22515,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_03</v>
       </c>
     </row>
-    <row r="280" xml:space="preserve">
+    <row r="280" xml:space="preserve" outlineLevel="1">
       <c r="A280" s="5" t="str">
         <v>AML_MSB002_MND_04</v>
       </c>
@@ -22588,7 +22591,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_04</v>
       </c>
     </row>
-    <row r="281" xml:space="preserve">
+    <row r="281" xml:space="preserve" outlineLevel="1">
       <c r="A281" s="5" t="str">
         <v>AML_MSB002_MND_05</v>
       </c>
@@ -22664,7 +22667,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_05</v>
       </c>
     </row>
-    <row r="282" xml:space="preserve">
+    <row r="282" xml:space="preserve" outlineLevel="1">
       <c r="A282" s="5" t="str">
         <v>AML_MSB002_MND_06</v>
       </c>
@@ -22740,7 +22743,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_06</v>
       </c>
     </row>
-    <row r="283" xml:space="preserve">
+    <row r="283" xml:space="preserve" outlineLevel="1">
       <c r="A283" s="5" t="str">
         <v>AML_MSB002_MND_07</v>
       </c>
@@ -22816,7 +22819,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_07</v>
       </c>
     </row>
-    <row r="284" xml:space="preserve">
+    <row r="284" xml:space="preserve" outlineLevel="1">
       <c r="A284" s="5" t="str">
         <v>AML_MSB002_MND_08</v>
       </c>
@@ -22892,7 +22895,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_08</v>
       </c>
     </row>
-    <row r="285" xml:space="preserve">
+    <row r="285" xml:space="preserve" outlineLevel="1">
       <c r="A285" s="5" t="str">
         <v>AML_MSB002_MND_09</v>
       </c>
@@ -22968,7 +22971,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_09</v>
       </c>
     </row>
-    <row r="286" xml:space="preserve">
+    <row r="286" xml:space="preserve" outlineLevel="1">
       <c r="A286" s="5" t="str">
         <v>AML_MSB002_MND_10</v>
       </c>
@@ -23044,7 +23047,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_10</v>
       </c>
     </row>
-    <row r="287" xml:space="preserve">
+    <row r="287" xml:space="preserve" outlineLevel="1">
       <c r="A287" s="5" t="str">
         <v>AML_MSB002_MND_11</v>
       </c>
@@ -23120,7 +23123,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_11</v>
       </c>
     </row>
-    <row r="288" xml:space="preserve">
+    <row r="288" xml:space="preserve" outlineLevel="1">
       <c r="A288" s="5" t="str">
         <v>AML_MSB002_MND_12</v>
       </c>
@@ -23196,7 +23199,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_12</v>
       </c>
     </row>
-    <row r="289" xml:space="preserve">
+    <row r="289" xml:space="preserve" outlineLevel="1">
       <c r="A289" s="5" t="str">
         <v>AML_MSB002_MND_13</v>
       </c>
@@ -23272,7 +23275,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_13</v>
       </c>
     </row>
-    <row r="290" xml:space="preserve">
+    <row r="290" xml:space="preserve" outlineLevel="1">
       <c r="A290" s="5" t="str">
         <v>AML_MSB002_MND_14</v>
       </c>
@@ -23348,7 +23351,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_14</v>
       </c>
     </row>
-    <row r="291" xml:space="preserve">
+    <row r="291" xml:space="preserve" outlineLevel="1">
       <c r="A291" s="5" t="str">
         <v>AML_MSB002_MND_15</v>
       </c>
@@ -23424,7 +23427,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_15</v>
       </c>
     </row>
-    <row r="292" xml:space="preserve">
+    <row r="292" xml:space="preserve" outlineLevel="1">
       <c r="A292" s="5" t="str">
         <v>AML_MSB002_MND_16</v>
       </c>
@@ -23500,7 +23503,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_16</v>
       </c>
     </row>
-    <row r="293" xml:space="preserve">
+    <row r="293" xml:space="preserve" outlineLevel="1">
       <c r="A293" s="5" t="str">
         <v>AML_MSB002_MND_17</v>
       </c>
@@ -23576,7 +23579,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_17</v>
       </c>
     </row>
-    <row r="294" xml:space="preserve">
+    <row r="294" xml:space="preserve" outlineLevel="1">
       <c r="A294" s="5" t="str">
         <v>AML_MSB002_MND_18</v>
       </c>
@@ -23652,7 +23655,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_18</v>
       </c>
     </row>
-    <row r="295" xml:space="preserve">
+    <row r="295" xml:space="preserve" outlineLevel="1">
       <c r="A295" s="5" t="str">
         <v>AML_MSB002_MND_19</v>
       </c>
@@ -23728,7 +23731,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_19</v>
       </c>
     </row>
-    <row r="296" xml:space="preserve">
+    <row r="296" xml:space="preserve" outlineLevel="1">
       <c r="A296" s="5" t="str">
         <v>AML_MSB002_MND_20</v>
       </c>
@@ -23804,7 +23807,7 @@
         <v>TD: TD_P2_043 | [GIU NGUYEN] ID goc: AML_MSB002_MND_20</v>
       </c>
     </row>
-    <row r="297" xml:space="preserve">
+    <row r="297" xml:space="preserve" outlineLevel="1">
       <c r="A297" s="5" t="str">
         <v>AML_MSB002_MND_21</v>
       </c>
@@ -23939,7 +23942,7 @@
         <v/>
       </c>
     </row>
-    <row r="299" xml:space="preserve">
+    <row r="299" xml:space="preserve" outlineLevel="1">
       <c r="A299" s="5" t="str">
         <v>AML_MSB003_MND_33</v>
       </c>
@@ -24015,7 +24018,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_33</v>
       </c>
     </row>
-    <row r="300" xml:space="preserve">
+    <row r="300" xml:space="preserve" outlineLevel="1">
       <c r="A300" s="5" t="str">
         <v>AML_MSB003_MND_34</v>
       </c>
@@ -24150,7 +24153,7 @@
         <v/>
       </c>
     </row>
-    <row r="302" xml:space="preserve">
+    <row r="302" xml:space="preserve" outlineLevel="1">
       <c r="A302" s="5" t="str">
         <v>AML_MSB003_MND_05</v>
       </c>
@@ -24226,7 +24229,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_05</v>
       </c>
     </row>
-    <row r="303" xml:space="preserve">
+    <row r="303" xml:space="preserve" outlineLevel="1">
       <c r="A303" s="5" t="str">
         <v>AML_MSB003_MND_06</v>
       </c>
@@ -24302,7 +24305,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_06</v>
       </c>
     </row>
-    <row r="304" xml:space="preserve">
+    <row r="304" xml:space="preserve" outlineLevel="1">
       <c r="A304" s="5" t="str">
         <v>AML_MSB003_MND_07</v>
       </c>
@@ -24437,7 +24440,7 @@
         <v/>
       </c>
     </row>
-    <row r="306" xml:space="preserve">
+    <row r="306" xml:space="preserve" outlineLevel="1">
       <c r="A306" s="5" t="str">
         <v>AML_MSB003_MND_02</v>
       </c>
@@ -24513,7 +24516,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_02</v>
       </c>
     </row>
-    <row r="307" xml:space="preserve">
+    <row r="307" xml:space="preserve" outlineLevel="1">
       <c r="A307" s="5" t="str">
         <v>AML_MSB003_MND_03</v>
       </c>
@@ -24589,7 +24592,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_03</v>
       </c>
     </row>
-    <row r="308" xml:space="preserve">
+    <row r="308" xml:space="preserve" outlineLevel="1">
       <c r="A308" s="5" t="str">
         <v>AML_MSB003_MND_04</v>
       </c>
@@ -24724,7 +24727,7 @@
         <v/>
       </c>
     </row>
-    <row r="310" xml:space="preserve">
+    <row r="310" xml:space="preserve" outlineLevel="1">
       <c r="A310" s="5" t="str">
         <v>AML_MSB003_MND_44</v>
       </c>
@@ -24800,7 +24803,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_44</v>
       </c>
     </row>
-    <row r="311" xml:space="preserve">
+    <row r="311" xml:space="preserve" outlineLevel="1">
       <c r="A311" s="5" t="str">
         <v>AML_MSB003_MND_45</v>
       </c>
@@ -24935,7 +24938,7 @@
         <v/>
       </c>
     </row>
-    <row r="313" xml:space="preserve">
+    <row r="313" xml:space="preserve" outlineLevel="1">
       <c r="A313" s="5" t="str">
         <v>AML_MSB003_MND_35</v>
       </c>
@@ -25011,7 +25014,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_35</v>
       </c>
     </row>
-    <row r="314" xml:space="preserve">
+    <row r="314" xml:space="preserve" outlineLevel="1">
       <c r="A314" s="5" t="str">
         <v>AML_MSB003_MND_36</v>
       </c>
@@ -25087,7 +25090,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_36</v>
       </c>
     </row>
-    <row r="315" xml:space="preserve">
+    <row r="315" xml:space="preserve" outlineLevel="1">
       <c r="A315" s="5" t="str">
         <v>AML_MSB003_MND_37</v>
       </c>
@@ -25163,7 +25166,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_37</v>
       </c>
     </row>
-    <row r="316" xml:space="preserve">
+    <row r="316" xml:space="preserve" outlineLevel="1">
       <c r="A316" s="5" t="str">
         <v>AML_MSB003_MND_38</v>
       </c>
@@ -25239,7 +25242,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_38</v>
       </c>
     </row>
-    <row r="317" xml:space="preserve">
+    <row r="317" xml:space="preserve" outlineLevel="1">
       <c r="A317" s="5" t="str">
         <v>AML_MSB003_MND_39</v>
       </c>
@@ -25315,7 +25318,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_39</v>
       </c>
     </row>
-    <row r="318" xml:space="preserve">
+    <row r="318" xml:space="preserve" outlineLevel="1">
       <c r="A318" s="5" t="str">
         <v>AML_MSB003_MND_40</v>
       </c>
@@ -25391,7 +25394,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_40</v>
       </c>
     </row>
-    <row r="319" xml:space="preserve">
+    <row r="319" xml:space="preserve" outlineLevel="1">
       <c r="A319" s="5" t="str">
         <v>AML_MSB003_MND_41</v>
       </c>
@@ -25467,7 +25470,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_41</v>
       </c>
     </row>
-    <row r="320" xml:space="preserve">
+    <row r="320" xml:space="preserve" outlineLevel="1">
       <c r="A320" s="5" t="str">
         <v>AML_MSB003_MND_42</v>
       </c>
@@ -25543,7 +25546,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_42</v>
       </c>
     </row>
-    <row r="321" xml:space="preserve">
+    <row r="321" xml:space="preserve" outlineLevel="1">
       <c r="A321" s="5" t="str">
         <v>AML_MSB003_MND_43</v>
       </c>
@@ -25678,7 +25681,7 @@
         <v/>
       </c>
     </row>
-    <row r="323" xml:space="preserve">
+    <row r="323" xml:space="preserve" outlineLevel="1">
       <c r="A323" s="5" t="str">
         <v>AML_MSB003_MND_08</v>
       </c>
@@ -25754,7 +25757,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_08</v>
       </c>
     </row>
-    <row r="324" xml:space="preserve">
+    <row r="324" xml:space="preserve" outlineLevel="1">
       <c r="A324" s="5" t="str">
         <v>AML_MSB003_MND_09</v>
       </c>
@@ -25830,7 +25833,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_09</v>
       </c>
     </row>
-    <row r="325" xml:space="preserve">
+    <row r="325" xml:space="preserve" outlineLevel="1">
       <c r="A325" s="5" t="str">
         <v>AML_MSB003_MND_10</v>
       </c>
@@ -25906,7 +25909,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_10</v>
       </c>
     </row>
-    <row r="326" xml:space="preserve">
+    <row r="326" xml:space="preserve" outlineLevel="1">
       <c r="A326" s="5" t="str">
         <v>AML_MSB003_MND_11</v>
       </c>
@@ -25982,7 +25985,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_11</v>
       </c>
     </row>
-    <row r="327" xml:space="preserve">
+    <row r="327" xml:space="preserve" outlineLevel="1">
       <c r="A327" s="5" t="str">
         <v>AML_MSB003_MND_12</v>
       </c>
@@ -26058,7 +26061,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_12</v>
       </c>
     </row>
-    <row r="328" xml:space="preserve">
+    <row r="328" xml:space="preserve" outlineLevel="1">
       <c r="A328" s="5" t="str">
         <v>AML_MSB003_MND_13</v>
       </c>
@@ -26134,7 +26137,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_13</v>
       </c>
     </row>
-    <row r="329" xml:space="preserve">
+    <row r="329" xml:space="preserve" outlineLevel="1">
       <c r="A329" s="5" t="str">
         <v>AML_MSB003_MND_14</v>
       </c>
@@ -26210,7 +26213,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_14</v>
       </c>
     </row>
-    <row r="330" xml:space="preserve">
+    <row r="330" xml:space="preserve" outlineLevel="1">
       <c r="A330" s="5" t="str">
         <v>AML_MSB003_MND_15</v>
       </c>
@@ -26286,7 +26289,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_15</v>
       </c>
     </row>
-    <row r="331" xml:space="preserve">
+    <row r="331" xml:space="preserve" outlineLevel="1">
       <c r="A331" s="5" t="str">
         <v>AML_MSB003_MND_16</v>
       </c>
@@ -26362,7 +26365,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_16</v>
       </c>
     </row>
-    <row r="332" xml:space="preserve">
+    <row r="332" xml:space="preserve" outlineLevel="1">
       <c r="A332" s="5" t="str">
         <v>AML_MSB003_MND_17</v>
       </c>
@@ -26438,7 +26441,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_17</v>
       </c>
     </row>
-    <row r="333" xml:space="preserve">
+    <row r="333" xml:space="preserve" outlineLevel="1">
       <c r="A333" s="5" t="str">
         <v>AML_MSB003_MND_18</v>
       </c>
@@ -26514,7 +26517,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_18</v>
       </c>
     </row>
-    <row r="334" xml:space="preserve">
+    <row r="334" xml:space="preserve" outlineLevel="1">
       <c r="A334" s="5" t="str">
         <v>AML_MSB003_MND_19</v>
       </c>
@@ -26590,7 +26593,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_19</v>
       </c>
     </row>
-    <row r="335" xml:space="preserve">
+    <row r="335" xml:space="preserve" outlineLevel="1">
       <c r="A335" s="5" t="str">
         <v>AML_MSB003_MND_20</v>
       </c>
@@ -26666,7 +26669,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_20</v>
       </c>
     </row>
-    <row r="336" xml:space="preserve">
+    <row r="336" xml:space="preserve" outlineLevel="1">
       <c r="A336" s="5" t="str">
         <v>AML_MSB003_MND_21</v>
       </c>
@@ -26742,7 +26745,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_21</v>
       </c>
     </row>
-    <row r="337" xml:space="preserve">
+    <row r="337" xml:space="preserve" outlineLevel="1">
       <c r="A337" s="5" t="str">
         <v>AML_MSB003_MND_22</v>
       </c>
@@ -26818,7 +26821,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_22</v>
       </c>
     </row>
-    <row r="338" xml:space="preserve">
+    <row r="338" xml:space="preserve" outlineLevel="1">
       <c r="A338" s="5" t="str">
         <v>AML_MSB003_MND_23</v>
       </c>
@@ -26894,7 +26897,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_23</v>
       </c>
     </row>
-    <row r="339" xml:space="preserve">
+    <row r="339" xml:space="preserve" outlineLevel="1">
       <c r="A339" s="5" t="str">
         <v>AML_MSB003_MND_24</v>
       </c>
@@ -26970,7 +26973,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_24</v>
       </c>
     </row>
-    <row r="340" xml:space="preserve">
+    <row r="340" xml:space="preserve" outlineLevel="1">
       <c r="A340" s="5" t="str">
         <v>AML_MSB003_MND_25</v>
       </c>
@@ -27046,7 +27049,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_25</v>
       </c>
     </row>
-    <row r="341" xml:space="preserve">
+    <row r="341" xml:space="preserve" outlineLevel="1">
       <c r="A341" s="5" t="str">
         <v>AML_MSB003_MND_26</v>
       </c>
@@ -27122,7 +27125,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_26</v>
       </c>
     </row>
-    <row r="342" xml:space="preserve">
+    <row r="342" xml:space="preserve" outlineLevel="1">
       <c r="A342" s="5" t="str">
         <v>AML_MSB003_MND_27</v>
       </c>
@@ -27198,7 +27201,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_27</v>
       </c>
     </row>
-    <row r="343" xml:space="preserve">
+    <row r="343" xml:space="preserve" outlineLevel="1">
       <c r="A343" s="5" t="str">
         <v>AML_MSB003_MND_28</v>
       </c>
@@ -27274,7 +27277,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_28</v>
       </c>
     </row>
-    <row r="344" xml:space="preserve">
+    <row r="344" xml:space="preserve" outlineLevel="1">
       <c r="A344" s="5" t="str">
         <v>AML_MSB003_MND_29</v>
       </c>
@@ -27350,7 +27353,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_29</v>
       </c>
     </row>
-    <row r="345" xml:space="preserve">
+    <row r="345" xml:space="preserve" outlineLevel="1">
       <c r="A345" s="5" t="str">
         <v>AML_MSB003_MND_30</v>
       </c>
@@ -27426,7 +27429,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_30</v>
       </c>
     </row>
-    <row r="346" xml:space="preserve">
+    <row r="346" xml:space="preserve" outlineLevel="1">
       <c r="A346" s="5" t="str">
         <v>AML_MSB003_MND_31</v>
       </c>
@@ -27502,7 +27505,7 @@
         <v>TD: TD_P2_047 | [GIU NGUYEN] ID goc: AML_MSB003_MND_31</v>
       </c>
     </row>
-    <row r="347" xml:space="preserve">
+    <row r="347" xml:space="preserve" outlineLevel="1">
       <c r="A347" s="5" t="str">
         <v>AML_MSB003_MND_32</v>
       </c>
@@ -27637,7 +27640,7 @@
         <v/>
       </c>
     </row>
-    <row r="349" xml:space="preserve">
+    <row r="349" xml:space="preserve" outlineLevel="1">
       <c r="A349" s="5" t="str">
         <v>AML_MSB003_MND_01</v>
       </c>
@@ -27771,7 +27774,7 @@
         <v/>
       </c>
     </row>
-    <row r="351" xml:space="preserve">
+    <row r="351" xml:space="preserve" outlineLevel="1">
       <c r="A351" s="5" t="str">
         <v>AML_API_HTTP_03</v>
       </c>
@@ -27851,7 +27854,7 @@
         <v>TD: TD_P1_017 | [GIU NGUYEN] ID goc: AML_API_HTTP_03</v>
       </c>
     </row>
-    <row r="352" xml:space="preserve">
+    <row r="352" xml:space="preserve" outlineLevel="1">
       <c r="A352" s="5" t="str">
         <v/>
       </c>
@@ -27927,7 +27930,7 @@
         <v>TD: TD_P1_018 | [TC MOI THEM] [Security] | Ly do: TC goc chi kiem truong hop THIEU Authorization (AML_API_HTTP_03), chua kiem truong hop co Authorization nhung sai credential</v>
       </c>
     </row>
-    <row r="353" xml:space="preserve">
+    <row r="353" xml:space="preserve" outlineLevel="1">
       <c r="A353" s="5" t="str">
         <v/>
       </c>
@@ -28061,7 +28064,7 @@
         <v/>
       </c>
     </row>
-    <row r="355" xml:space="preserve">
+    <row r="355" xml:space="preserve" outlineLevel="1">
       <c r="A355" s="5" t="str">
         <v>AML_API_HDR_09</v>
       </c>
@@ -28142,7 +28145,7 @@
         <v>TD: TD_P3_001 | [GIU NGUYEN] ID goc: AML_API_HDR_09</v>
       </c>
     </row>
-    <row r="356" xml:space="preserve">
+    <row r="356" xml:space="preserve" outlineLevel="1">
       <c r="A356" s="5" t="str">
         <v>AML_API_HDR_10</v>
       </c>
@@ -28230,7 +28233,7 @@
         <v>TD: TD_P3_002 | [GIU NGUYEN] ID goc: AML_API_HDR_10</v>
       </c>
     </row>
-    <row r="357" xml:space="preserve">
+    <row r="357" xml:space="preserve" outlineLevel="1">
       <c r="A357" s="5" t="str">
         <v/>
       </c>
@@ -28313,7 +28316,7 @@
         <v>TD: TD_P3_003 | [TC MOI THEM] [ST] | Ly do: TC goc co case isCallBack=Y thanh cong (AML_API_HDR_09, AML_API_MT_07) nhung chua co case callback that bai</v>
       </c>
     </row>
-    <row r="358" xml:space="preserve">
+    <row r="358" xml:space="preserve" outlineLevel="1">
       <c r="A358" s="5" t="str">
         <v>AML_API_NF_04</v>
       </c>
@@ -28391,7 +28394,7 @@
         <v>TD: TD_P3_004 | [GIU NGUYEN] ID goc: AML_API_NF_04</v>
       </c>
     </row>
-    <row r="359" xml:space="preserve">
+    <row r="359" xml:space="preserve" outlineLevel="1">
       <c r="A359" s="5" t="str">
         <v>AML_API_MT_06</v>
       </c>
@@ -28469,7 +28472,7 @@
         <v>TD: TD_P3_016 | [GIU NGUYEN] ID goc: AML_API_MT_06</v>
       </c>
     </row>
-    <row r="360" xml:space="preserve">
+    <row r="360" xml:space="preserve" outlineLevel="1">
       <c r="A360" s="5" t="str">
         <v>AML_API_MT_07</v>
       </c>
@@ -28613,7 +28616,7 @@
         <v/>
       </c>
     </row>
-    <row r="362" xml:space="preserve">
+    <row r="362" xml:space="preserve" outlineLevel="1">
       <c r="A362" s="5" t="str">
         <v>AML_API_RESP_01</v>
       </c>
@@ -28705,7 +28708,7 @@
         <v>TD: TD_P4_001 | [GIU NGUYEN] ID goc: AML_API_RESP_01</v>
       </c>
     </row>
-    <row r="363" xml:space="preserve">
+    <row r="363" xml:space="preserve" outlineLevel="1">
       <c r="A363" s="5" t="str">
         <v>AML_API_RESP_02</v>
       </c>
@@ -28797,7 +28800,7 @@
         <v>TD: TD_P4_002 | [GIU NGUYEN] ID goc: AML_API_RESP_02</v>
       </c>
     </row>
-    <row r="364" xml:space="preserve">
+    <row r="364" xml:space="preserve" outlineLevel="1">
       <c r="A364" s="5" t="str">
         <v>AML_API_RESP_03</v>
       </c>
@@ -28889,7 +28892,7 @@
         <v>TD: TD_P4_003 | [GIU NGUYEN] ID goc: AML_API_RESP_03</v>
       </c>
     </row>
-    <row r="365" xml:space="preserve">
+    <row r="365" xml:space="preserve" outlineLevel="1">
       <c r="A365" s="5" t="str">
         <v>AML_API_RESP_04</v>
       </c>
@@ -28968,7 +28971,7 @@
         <v>TD: TD_P4_004 | [GIU NGUYEN] ID goc: AML_API_RESP_04</v>
       </c>
     </row>
-    <row r="366" xml:space="preserve">
+    <row r="366" xml:space="preserve" outlineLevel="1">
       <c r="A366" s="5" t="str">
         <v>AML_API_NF_05</v>
       </c>
@@ -29041,7 +29044,7 @@
         <v>TD: TD_P4_004 | [GIU NGUYEN] ID goc: AML_API_NF_05</v>
       </c>
     </row>
-    <row r="367" xml:space="preserve">
+    <row r="367" xml:space="preserve" outlineLevel="1">
       <c r="A367" s="5" t="str">
         <v>AML_API_RESP_08</v>
       </c>
@@ -29122,7 +29125,7 @@
         <v>TD: TD_P4_005 | [GIU NGUYEN] ID goc: AML_API_RESP_08</v>
       </c>
     </row>
-    <row r="368" xml:space="preserve">
+    <row r="368" xml:space="preserve" outlineLevel="1">
       <c r="A368" s="5" t="str">
         <v/>
       </c>
@@ -29199,7 +29202,7 @@
         <v>TD: TD_P4_006 | [TC MOI THEM] [RSP-Schema] | Ly do: Contract verification - TC goc kiem "day du 12 field" (AML_API_RESP_01) nhung chua kiem chieu nguoc lai la khong co field thua</v>
       </c>
     </row>
-    <row r="369" xml:space="preserve">
+    <row r="369" xml:space="preserve" outlineLevel="1">
       <c r="A369" s="5" t="str">
         <v/>
       </c>
@@ -29333,7 +29336,7 @@
         <v/>
       </c>
     </row>
-    <row r="371" xml:space="preserve">
+    <row r="371" xml:space="preserve" outlineLevel="1">
       <c r="A371" s="5" t="str">
         <v>AML_API_RESP_06</v>
       </c>
@@ -29415,7 +29418,7 @@
         <v>TD: TD_P4_008 | [GIU NGUYEN] ID goc: AML_API_RESP_06</v>
       </c>
     </row>
-    <row r="372" xml:space="preserve">
+    <row r="372" xml:space="preserve" outlineLevel="1">
       <c r="A372" s="5" t="str">
         <v>AML_API_RESP_07</v>
       </c>
@@ -29498,7 +29501,7 @@
         <v>TD: TD_P4_009 | [GIU NGUYEN] ID goc: AML_API_RESP_07</v>
       </c>
     </row>
-    <row r="373" xml:space="preserve">
+    <row r="373" xml:space="preserve" outlineLevel="1">
       <c r="A373" s="5" t="str">
         <v>AML_API_RESP_09</v>
       </c>
@@ -29578,7 +29581,7 @@
         <v>TD: TD_P4_010 | [GIU NGUYEN] ID goc: AML_API_RESP_09</v>
       </c>
     </row>
-    <row r="374" xml:space="preserve">
+    <row r="374" xml:space="preserve" outlineLevel="1">
       <c r="A374" s="5" t="str">
         <v>AML_API_RESP_10</v>
       </c>
@@ -29658,7 +29661,7 @@
         <v>TD: TD_P4_011 | [GIU NGUYEN] ID goc: AML_API_RESP_10</v>
       </c>
     </row>
-    <row r="375" xml:space="preserve">
+    <row r="375" xml:space="preserve" outlineLevel="1">
       <c r="A375" s="5" t="str">
         <v/>
       </c>
@@ -29786,7 +29789,7 @@
         <v/>
       </c>
     </row>
-    <row r="377" xml:space="preserve">
+    <row r="377" xml:space="preserve" outlineLevel="1">
       <c r="A377" s="5" t="str">
         <v>AML_API_ERR_01</v>
       </c>
@@ -29870,7 +29873,7 @@
         <v>TD: TD_P4_013 | [GIU NGUYEN] ID goc: AML_API_ERR_01</v>
       </c>
     </row>
-    <row r="378" xml:space="preserve">
+    <row r="378" xml:space="preserve" outlineLevel="1">
       <c r="A378" s="5" t="str">
         <v>AML_API_ERR_02</v>
       </c>
@@ -29956,7 +29959,7 @@
         <v>TD: TD_P4_014 | [GIU NGUYEN] ID goc: AML_API_ERR_02</v>
       </c>
     </row>
-    <row r="379" xml:space="preserve">
+    <row r="379" xml:space="preserve" outlineLevel="1">
       <c r="A379" s="5" t="str">
         <v>AML_API_ERR_03</v>
       </c>
@@ -30031,7 +30034,7 @@
         <v>TD: TD_P4_015 | [GIU NGUYEN] ID goc: AML_API_ERR_03</v>
       </c>
     </row>
-    <row r="380" xml:space="preserve">
+    <row r="380" xml:space="preserve" outlineLevel="1">
       <c r="A380" s="5" t="str">
         <v>AML_API_ERR_04</v>
       </c>
@@ -30118,7 +30121,7 @@
         <v>TD: TD_P4_016 | [GIU NGUYEN] ID goc: AML_API_ERR_04</v>
       </c>
     </row>
-    <row r="381" xml:space="preserve">
+    <row r="381" xml:space="preserve" outlineLevel="1">
       <c r="A381" s="5" t="str">
         <v>AML_API_ERR_05</v>
       </c>
@@ -30205,7 +30208,7 @@
         <v>TD: TD_P4_017 | [GIU NGUYEN] ID goc: AML_API_ERR_05</v>
       </c>
     </row>
-    <row r="382" xml:space="preserve">
+    <row r="382" xml:space="preserve" outlineLevel="1">
       <c r="A382" s="5" t="str">
         <v>AML_API_ERR_06</v>
       </c>
@@ -30292,7 +30295,7 @@
         <v>TD: TD_P4_018 | [GIU NGUYEN] ID goc: AML_API_ERR_06</v>
       </c>
     </row>
-    <row r="383" xml:space="preserve">
+    <row r="383" xml:space="preserve" outlineLevel="1">
       <c r="A383" s="5" t="str">
         <v>AML_API_RESP_05</v>
       </c>
@@ -30365,7 +30368,7 @@
         <v>TD: TD_P4_019 | [GIU NGUYEN] ID goc: AML_API_RESP_05</v>
       </c>
     </row>
-    <row r="384" xml:space="preserve">
+    <row r="384" xml:space="preserve" outlineLevel="1">
       <c r="A384" s="5" t="str">
         <v>AML_API_HTTP_01</v>
       </c>
@@ -30447,7 +30450,7 @@
         <v>TD: TD_P4_019 | [GIU NGUYEN] ID goc: AML_API_HTTP_01</v>
       </c>
     </row>
-    <row r="385" xml:space="preserve">
+    <row r="385" xml:space="preserve" outlineLevel="1">
       <c r="A385" s="5" t="str">
         <v>AML_API_HTTP_02</v>
       </c>
@@ -30520,7 +30523,7 @@
         <v>TD: TD_P4_020 | [GIU NGUYEN] ID goc: AML_API_HTTP_02</v>
       </c>
     </row>
-    <row r="386" xml:space="preserve">
+    <row r="386" xml:space="preserve" outlineLevel="1">
       <c r="A386" s="5" t="str">
         <v>AML_API_HTTP_05</v>
       </c>
@@ -30598,7 +30601,7 @@
         <v>TD: TD_P4_021 | [GIU NGUYEN] ID goc: AML_API_HTTP_05</v>
       </c>
     </row>
-    <row r="387" xml:space="preserve">
+    <row r="387" xml:space="preserve" outlineLevel="1">
       <c r="A387" s="5" t="str">
         <v/>
       </c>

</xml_diff>